<commit_message>
Compléter à 184 prescripteurs avec les derniers nouveaux (DrName)
- 24 prescripteurs CORE récupérés depuis l'historique (suppression des 70)
- Noms analysés selon les mêmes règles (FIRST=prénom, LAST=nom)
- Numéros tous uniques, SR NO 1..184 (99 CORE, 85 NON CORE)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alpha_Kebe liste des prescripteur.xlsx
+++ b/Alpha_Kebe liste des prescripteur.xlsx
@@ -52293,32 +52293,97 @@
       <c r="IK162" s="43" t="n"/>
     </row>
     <row r="163" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A163" s="43" t="n"/>
-      <c r="C163" s="43" t="n"/>
-      <c r="D163" s="43" t="n"/>
-      <c r="E163" s="43" t="n"/>
-      <c r="F163" s="43" t="inlineStr">
+      <c r="A163" s="48" t="n">
+        <v>161</v>
+      </c>
+      <c r="B163" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C163" s="50" t="n"/>
+      <c r="D163" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E163" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F163" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G163" s="43" t="n"/>
-      <c r="H163" s="43" t="n"/>
-      <c r="I163" s="43" t="n"/>
-      <c r="J163" s="43" t="n"/>
-      <c r="K163" s="43" t="n"/>
-      <c r="L163" s="43" t="n"/>
-      <c r="O163" s="43" t="n"/>
-      <c r="P163" s="43" t="n"/>
-      <c r="Q163" s="43" t="n"/>
-      <c r="R163" s="43" t="n"/>
-      <c r="S163" s="43" t="n"/>
-      <c r="T163" s="43" t="n"/>
-      <c r="U163" s="43" t="n"/>
-      <c r="V163" s="43" t="n"/>
-      <c r="W163" s="43" t="n"/>
-      <c r="X163" s="43" t="n"/>
-      <c r="Y163" s="43" t="n"/>
+      <c r="G163" s="49" t="n"/>
+      <c r="H163" s="51" t="inlineStr">
+        <is>
+          <t>Amadou</t>
+        </is>
+      </c>
+      <c r="I163" s="51" t="inlineStr">
+        <is>
+          <t>Dia</t>
+        </is>
+      </c>
+      <c r="J163" s="51" t="inlineStr">
+        <is>
+          <t>Amadou Dia</t>
+        </is>
+      </c>
+      <c r="K163" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L163" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M163" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N163" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O163" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P163" s="51" t="inlineStr">
+        <is>
+          <t>Csref I</t>
+        </is>
+      </c>
+      <c r="Q163" s="54" t="n"/>
+      <c r="R163" s="55" t="inlineStr">
+        <is>
+          <t>71226650</t>
+        </is>
+      </c>
+      <c r="S163" s="55" t="n"/>
+      <c r="T163" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U163" s="65" t="n"/>
+      <c r="V163" s="57" t="n"/>
+      <c r="W163" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X163" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y163" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z163" s="43" t="n"/>
       <c r="AA163" s="43" t="n"/>
       <c r="AB163" s="43" t="n"/>
@@ -52541,32 +52606,97 @@
       <c r="IK163" s="43" t="n"/>
     </row>
     <row r="164" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A164" s="43" t="n"/>
-      <c r="C164" s="43" t="n"/>
-      <c r="D164" s="43" t="n"/>
-      <c r="E164" s="43" t="n"/>
-      <c r="F164" s="43" t="inlineStr">
+      <c r="A164" s="48" t="n">
+        <v>162</v>
+      </c>
+      <c r="B164" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C164" s="50" t="n"/>
+      <c r="D164" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E164" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F164" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G164" s="43" t="n"/>
-      <c r="H164" s="43" t="n"/>
-      <c r="I164" s="43" t="n"/>
-      <c r="J164" s="43" t="n"/>
-      <c r="K164" s="43" t="n"/>
-      <c r="L164" s="43" t="n"/>
-      <c r="O164" s="43" t="n"/>
-      <c r="P164" s="43" t="n"/>
-      <c r="Q164" s="43" t="n"/>
-      <c r="R164" s="43" t="n"/>
-      <c r="S164" s="43" t="n"/>
-      <c r="T164" s="43" t="n"/>
-      <c r="U164" s="43" t="n"/>
-      <c r="V164" s="43" t="n"/>
-      <c r="W164" s="43" t="n"/>
-      <c r="X164" s="43" t="n"/>
-      <c r="Y164" s="43" t="n"/>
+      <c r="G164" s="49" t="n"/>
+      <c r="H164" s="51" t="inlineStr">
+        <is>
+          <t>Fatoumata</t>
+        </is>
+      </c>
+      <c r="I164" s="51" t="inlineStr">
+        <is>
+          <t>Diabate</t>
+        </is>
+      </c>
+      <c r="J164" s="51" t="inlineStr">
+        <is>
+          <t>Fatoumata Diabate</t>
+        </is>
+      </c>
+      <c r="K164" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L164" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M164" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N164" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O164" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P164" s="51" t="inlineStr">
+        <is>
+          <t>Csref I</t>
+        </is>
+      </c>
+      <c r="Q164" s="54" t="n"/>
+      <c r="R164" s="55" t="inlineStr">
+        <is>
+          <t>72492457</t>
+        </is>
+      </c>
+      <c r="S164" s="55" t="n"/>
+      <c r="T164" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U164" s="65" t="n"/>
+      <c r="V164" s="57" t="n"/>
+      <c r="W164" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X164" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y164" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z164" s="43" t="n"/>
       <c r="AA164" s="43" t="n"/>
       <c r="AB164" s="43" t="n"/>
@@ -52789,32 +52919,97 @@
       <c r="IK164" s="43" t="n"/>
     </row>
     <row r="165" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A165" s="43" t="n"/>
-      <c r="C165" s="43" t="n"/>
-      <c r="D165" s="43" t="n"/>
-      <c r="E165" s="43" t="n"/>
-      <c r="F165" s="43" t="inlineStr">
+      <c r="A165" s="48" t="n">
+        <v>163</v>
+      </c>
+      <c r="B165" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C165" s="50" t="n"/>
+      <c r="D165" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E165" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F165" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G165" s="43" t="n"/>
-      <c r="H165" s="43" t="n"/>
-      <c r="I165" s="43" t="n"/>
-      <c r="J165" s="43" t="n"/>
-      <c r="K165" s="43" t="n"/>
-      <c r="L165" s="43" t="n"/>
-      <c r="O165" s="43" t="n"/>
-      <c r="P165" s="43" t="n"/>
-      <c r="Q165" s="43" t="n"/>
-      <c r="R165" s="43" t="n"/>
-      <c r="S165" s="43" t="n"/>
-      <c r="T165" s="43" t="n"/>
-      <c r="U165" s="43" t="n"/>
-      <c r="V165" s="43" t="n"/>
-      <c r="W165" s="43" t="n"/>
-      <c r="X165" s="43" t="n"/>
-      <c r="Y165" s="43" t="n"/>
+      <c r="G165" s="49" t="n"/>
+      <c r="H165" s="51" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="I165" s="51" t="inlineStr">
+        <is>
+          <t>Diabate</t>
+        </is>
+      </c>
+      <c r="J165" s="51" t="inlineStr">
+        <is>
+          <t>Daniel Diabate</t>
+        </is>
+      </c>
+      <c r="K165" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L165" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M165" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N165" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O165" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P165" s="51" t="inlineStr">
+        <is>
+          <t>Csref I</t>
+        </is>
+      </c>
+      <c r="Q165" s="54" t="n"/>
+      <c r="R165" s="55" t="inlineStr">
+        <is>
+          <t>79270108</t>
+        </is>
+      </c>
+      <c r="S165" s="55" t="n"/>
+      <c r="T165" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U165" s="65" t="n"/>
+      <c r="V165" s="57" t="n"/>
+      <c r="W165" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X165" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y165" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z165" s="43" t="n"/>
       <c r="AA165" s="43" t="n"/>
       <c r="AB165" s="43" t="n"/>
@@ -53037,32 +53232,97 @@
       <c r="IK165" s="43" t="n"/>
     </row>
     <row r="166" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A166" s="43" t="n"/>
-      <c r="C166" s="43" t="n"/>
-      <c r="D166" s="43" t="n"/>
-      <c r="E166" s="43" t="n"/>
-      <c r="F166" s="43" t="inlineStr">
+      <c r="A166" s="48" t="n">
+        <v>164</v>
+      </c>
+      <c r="B166" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C166" s="50" t="n"/>
+      <c r="D166" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E166" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F166" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G166" s="43" t="n"/>
-      <c r="H166" s="43" t="n"/>
-      <c r="I166" s="43" t="n"/>
-      <c r="J166" s="43" t="n"/>
-      <c r="K166" s="43" t="n"/>
-      <c r="L166" s="43" t="n"/>
-      <c r="O166" s="43" t="n"/>
-      <c r="P166" s="43" t="n"/>
-      <c r="Q166" s="43" t="n"/>
-      <c r="R166" s="43" t="n"/>
-      <c r="S166" s="43" t="n"/>
-      <c r="T166" s="43" t="n"/>
-      <c r="U166" s="43" t="n"/>
-      <c r="V166" s="43" t="n"/>
-      <c r="W166" s="43" t="n"/>
-      <c r="X166" s="43" t="n"/>
-      <c r="Y166" s="43" t="n"/>
+      <c r="G166" s="49" t="n"/>
+      <c r="H166" s="51" t="inlineStr">
+        <is>
+          <t>Moumoune</t>
+        </is>
+      </c>
+      <c r="I166" s="51" t="inlineStr">
+        <is>
+          <t>Tangara</t>
+        </is>
+      </c>
+      <c r="J166" s="51" t="inlineStr">
+        <is>
+          <t>Moumoune Tangara</t>
+        </is>
+      </c>
+      <c r="K166" s="52" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="L166" s="53" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="M166" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N166" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O166" s="51" t="inlineStr">
+        <is>
+          <t>Cmad</t>
+        </is>
+      </c>
+      <c r="P166" s="51" t="inlineStr">
+        <is>
+          <t>Cmad</t>
+        </is>
+      </c>
+      <c r="Q166" s="54" t="n"/>
+      <c r="R166" s="55" t="inlineStr">
+        <is>
+          <t>70234051</t>
+        </is>
+      </c>
+      <c r="S166" s="55" t="n"/>
+      <c r="T166" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U166" s="65" t="n"/>
+      <c r="V166" s="57" t="n"/>
+      <c r="W166" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X166" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y166" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z166" s="43" t="n"/>
       <c r="AA166" s="43" t="n"/>
       <c r="AB166" s="43" t="n"/>
@@ -53285,32 +53545,97 @@
       <c r="IK166" s="43" t="n"/>
     </row>
     <row r="167" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A167" s="43" t="n"/>
-      <c r="C167" s="43" t="n"/>
-      <c r="D167" s="43" t="n"/>
-      <c r="E167" s="43" t="n"/>
-      <c r="F167" s="43" t="inlineStr">
+      <c r="A167" s="48" t="n">
+        <v>165</v>
+      </c>
+      <c r="B167" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C167" s="50" t="n"/>
+      <c r="D167" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E167" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F167" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G167" s="43" t="n"/>
-      <c r="H167" s="43" t="n"/>
-      <c r="I167" s="43" t="n"/>
-      <c r="J167" s="43" t="n"/>
-      <c r="K167" s="43" t="n"/>
-      <c r="L167" s="43" t="n"/>
-      <c r="O167" s="43" t="n"/>
-      <c r="P167" s="43" t="n"/>
-      <c r="Q167" s="43" t="n"/>
-      <c r="R167" s="43" t="n"/>
-      <c r="S167" s="43" t="n"/>
-      <c r="T167" s="43" t="n"/>
-      <c r="U167" s="43" t="n"/>
-      <c r="V167" s="43" t="n"/>
-      <c r="W167" s="43" t="n"/>
-      <c r="X167" s="43" t="n"/>
-      <c r="Y167" s="43" t="n"/>
+      <c r="G167" s="49" t="n"/>
+      <c r="H167" s="51" t="inlineStr">
+        <is>
+          <t>Abdoul</t>
+        </is>
+      </c>
+      <c r="I167" s="51" t="inlineStr">
+        <is>
+          <t>Traore</t>
+        </is>
+      </c>
+      <c r="J167" s="51" t="inlineStr">
+        <is>
+          <t>Abdoul Traore</t>
+        </is>
+      </c>
+      <c r="K167" s="52" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="L167" s="53" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="M167" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N167" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O167" s="51" t="inlineStr">
+        <is>
+          <t>Cm</t>
+        </is>
+      </c>
+      <c r="P167" s="51" t="inlineStr">
+        <is>
+          <t>Cm Espoir</t>
+        </is>
+      </c>
+      <c r="Q167" s="54" t="n"/>
+      <c r="R167" s="55" t="inlineStr">
+        <is>
+          <t>92496479</t>
+        </is>
+      </c>
+      <c r="S167" s="55" t="n"/>
+      <c r="T167" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U167" s="65" t="n"/>
+      <c r="V167" s="57" t="n"/>
+      <c r="W167" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X167" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y167" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z167" s="43" t="n"/>
       <c r="AA167" s="43" t="n"/>
       <c r="AB167" s="43" t="n"/>
@@ -53533,32 +53858,97 @@
       <c r="IK167" s="43" t="n"/>
     </row>
     <row r="168" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A168" s="43" t="n"/>
-      <c r="C168" s="43" t="n"/>
-      <c r="D168" s="43" t="n"/>
-      <c r="E168" s="43" t="n"/>
-      <c r="F168" s="43" t="inlineStr">
+      <c r="A168" s="48" t="n">
+        <v>166</v>
+      </c>
+      <c r="B168" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C168" s="50" t="n"/>
+      <c r="D168" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E168" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F168" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G168" s="43" t="n"/>
-      <c r="H168" s="43" t="n"/>
-      <c r="I168" s="43" t="n"/>
-      <c r="J168" s="43" t="n"/>
-      <c r="K168" s="43" t="n"/>
-      <c r="L168" s="43" t="n"/>
-      <c r="O168" s="43" t="n"/>
-      <c r="P168" s="43" t="n"/>
-      <c r="Q168" s="43" t="n"/>
-      <c r="R168" s="43" t="n"/>
-      <c r="S168" s="43" t="n"/>
-      <c r="T168" s="43" t="n"/>
-      <c r="U168" s="43" t="n"/>
-      <c r="V168" s="43" t="n"/>
-      <c r="W168" s="43" t="n"/>
-      <c r="X168" s="43" t="n"/>
-      <c r="Y168" s="43" t="n"/>
+      <c r="G168" s="49" t="n"/>
+      <c r="H168" s="51" t="inlineStr">
+        <is>
+          <t>Haby</t>
+        </is>
+      </c>
+      <c r="I168" s="51" t="inlineStr">
+        <is>
+          <t>Bagayoko</t>
+        </is>
+      </c>
+      <c r="J168" s="51" t="inlineStr">
+        <is>
+          <t>Haby Bagayoko</t>
+        </is>
+      </c>
+      <c r="K168" s="52" t="inlineStr">
+        <is>
+          <t>MID WIFE</t>
+        </is>
+      </c>
+      <c r="L168" s="53" t="inlineStr">
+        <is>
+          <t>MID WIFE</t>
+        </is>
+      </c>
+      <c r="M168" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N168" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O168" s="51" t="inlineStr">
+        <is>
+          <t>CDanaya</t>
+        </is>
+      </c>
+      <c r="P168" s="51" t="inlineStr">
+        <is>
+          <t>CDanaya</t>
+        </is>
+      </c>
+      <c r="Q168" s="54" t="n"/>
+      <c r="R168" s="55" t="inlineStr">
+        <is>
+          <t>73092253</t>
+        </is>
+      </c>
+      <c r="S168" s="55" t="n"/>
+      <c r="T168" s="49" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="U168" s="65" t="n"/>
+      <c r="V168" s="57" t="n"/>
+      <c r="W168" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X168" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y168" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z168" s="43" t="n"/>
       <c r="AA168" s="43" t="n"/>
       <c r="AB168" s="43" t="n"/>
@@ -53781,32 +54171,97 @@
       <c r="IK168" s="43" t="n"/>
     </row>
     <row r="169" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A169" s="43" t="n"/>
-      <c r="C169" s="43" t="n"/>
-      <c r="D169" s="43" t="n"/>
-      <c r="E169" s="43" t="n"/>
-      <c r="F169" s="43" t="inlineStr">
+      <c r="A169" s="48" t="n">
+        <v>167</v>
+      </c>
+      <c r="B169" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C169" s="50" t="n"/>
+      <c r="D169" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E169" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F169" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G169" s="43" t="n"/>
-      <c r="H169" s="43" t="n"/>
-      <c r="I169" s="43" t="n"/>
-      <c r="J169" s="43" t="n"/>
-      <c r="K169" s="43" t="n"/>
-      <c r="L169" s="43" t="n"/>
-      <c r="O169" s="43" t="n"/>
-      <c r="P169" s="43" t="n"/>
-      <c r="Q169" s="43" t="n"/>
-      <c r="R169" s="43" t="n"/>
-      <c r="S169" s="43" t="n"/>
-      <c r="T169" s="43" t="n"/>
-      <c r="U169" s="43" t="n"/>
-      <c r="V169" s="43" t="n"/>
-      <c r="W169" s="43" t="n"/>
-      <c r="X169" s="43" t="n"/>
-      <c r="Y169" s="43" t="n"/>
+      <c r="G169" s="49" t="n"/>
+      <c r="H169" s="51" t="inlineStr">
+        <is>
+          <t>Kodio</t>
+        </is>
+      </c>
+      <c r="I169" s="51" t="inlineStr">
+        <is>
+          <t>Bourama</t>
+        </is>
+      </c>
+      <c r="J169" s="51" t="inlineStr">
+        <is>
+          <t>Kodio Bourama</t>
+        </is>
+      </c>
+      <c r="K169" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L169" s="53" t="inlineStr">
+        <is>
+          <t>RHEUMATOlOGIST</t>
+        </is>
+      </c>
+      <c r="M169" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N169" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O169" s="51" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="P169" s="51" t="inlineStr">
+        <is>
+          <t>Groupe Medical</t>
+        </is>
+      </c>
+      <c r="Q169" s="54" t="n"/>
+      <c r="R169" s="55" t="inlineStr">
+        <is>
+          <t>75791055</t>
+        </is>
+      </c>
+      <c r="S169" s="55" t="n"/>
+      <c r="T169" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U169" s="65" t="n"/>
+      <c r="V169" s="57" t="n"/>
+      <c r="W169" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X169" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y169" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z169" s="43" t="n"/>
       <c r="AA169" s="43" t="n"/>
       <c r="AB169" s="43" t="n"/>
@@ -54029,32 +54484,97 @@
       <c r="IK169" s="43" t="n"/>
     </row>
     <row r="170" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A170" s="43" t="n"/>
-      <c r="C170" s="43" t="n"/>
-      <c r="D170" s="43" t="n"/>
-      <c r="E170" s="43" t="n"/>
-      <c r="F170" s="43" t="inlineStr">
+      <c r="A170" s="48" t="n">
+        <v>168</v>
+      </c>
+      <c r="B170" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C170" s="50" t="n"/>
+      <c r="D170" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E170" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F170" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G170" s="43" t="n"/>
-      <c r="H170" s="43" t="n"/>
-      <c r="I170" s="43" t="n"/>
-      <c r="J170" s="43" t="n"/>
-      <c r="K170" s="43" t="n"/>
-      <c r="L170" s="43" t="n"/>
-      <c r="O170" s="43" t="n"/>
-      <c r="P170" s="43" t="n"/>
-      <c r="Q170" s="43" t="n"/>
-      <c r="R170" s="43" t="n"/>
-      <c r="S170" s="43" t="n"/>
-      <c r="T170" s="43" t="n"/>
-      <c r="U170" s="43" t="n"/>
-      <c r="V170" s="43" t="n"/>
-      <c r="W170" s="43" t="n"/>
-      <c r="X170" s="43" t="n"/>
-      <c r="Y170" s="43" t="n"/>
+      <c r="G170" s="49" t="n"/>
+      <c r="H170" s="51" t="inlineStr">
+        <is>
+          <t>Senou</t>
+        </is>
+      </c>
+      <c r="I170" s="51" t="inlineStr">
+        <is>
+          <t>Bakary</t>
+        </is>
+      </c>
+      <c r="J170" s="51" t="inlineStr">
+        <is>
+          <t>Senou Bakary</t>
+        </is>
+      </c>
+      <c r="K170" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L170" s="53" t="inlineStr">
+        <is>
+          <t>CARDIOLOGIST</t>
+        </is>
+      </c>
+      <c r="M170" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N170" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O170" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P170" s="51" t="inlineStr">
+        <is>
+          <t>Csref I</t>
+        </is>
+      </c>
+      <c r="Q170" s="54" t="n"/>
+      <c r="R170" s="55" t="inlineStr">
+        <is>
+          <t>75079655</t>
+        </is>
+      </c>
+      <c r="S170" s="55" t="n"/>
+      <c r="T170" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U170" s="65" t="n"/>
+      <c r="V170" s="57" t="n"/>
+      <c r="W170" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X170" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y170" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z170" s="43" t="n"/>
       <c r="AA170" s="43" t="n"/>
       <c r="AB170" s="43" t="n"/>
@@ -54277,32 +54797,97 @@
       <c r="IK170" s="43" t="n"/>
     </row>
     <row r="171" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A171" s="43" t="n"/>
-      <c r="C171" s="43" t="n"/>
-      <c r="D171" s="43" t="n"/>
-      <c r="E171" s="43" t="n"/>
-      <c r="F171" s="43" t="inlineStr">
+      <c r="A171" s="48" t="n">
+        <v>169</v>
+      </c>
+      <c r="B171" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C171" s="50" t="n"/>
+      <c r="D171" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E171" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F171" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G171" s="43" t="n"/>
-      <c r="H171" s="43" t="n"/>
-      <c r="I171" s="43" t="n"/>
-      <c r="J171" s="43" t="n"/>
-      <c r="K171" s="43" t="n"/>
-      <c r="L171" s="43" t="n"/>
-      <c r="O171" s="43" t="n"/>
-      <c r="P171" s="43" t="n"/>
-      <c r="Q171" s="43" t="n"/>
-      <c r="R171" s="43" t="n"/>
-      <c r="S171" s="43" t="n"/>
-      <c r="T171" s="43" t="n"/>
-      <c r="U171" s="43" t="n"/>
-      <c r="V171" s="43" t="n"/>
-      <c r="W171" s="43" t="n"/>
-      <c r="X171" s="43" t="n"/>
-      <c r="Y171" s="43" t="n"/>
+      <c r="G171" s="49" t="n"/>
+      <c r="H171" s="51" t="inlineStr">
+        <is>
+          <t>Aminata</t>
+        </is>
+      </c>
+      <c r="I171" s="51" t="inlineStr">
+        <is>
+          <t>Ballo</t>
+        </is>
+      </c>
+      <c r="J171" s="51" t="inlineStr">
+        <is>
+          <t>Aminata Ballo</t>
+        </is>
+      </c>
+      <c r="K171" s="52" t="inlineStr">
+        <is>
+          <t>MID WIFE</t>
+        </is>
+      </c>
+      <c r="L171" s="53" t="inlineStr">
+        <is>
+          <t>MID WIFE</t>
+        </is>
+      </c>
+      <c r="M171" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N171" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O171" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P171" s="51" t="inlineStr">
+        <is>
+          <t>Csref I</t>
+        </is>
+      </c>
+      <c r="Q171" s="54" t="n"/>
+      <c r="R171" s="55" t="inlineStr">
+        <is>
+          <t>66983505</t>
+        </is>
+      </c>
+      <c r="S171" s="55" t="n"/>
+      <c r="T171" s="49" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="U171" s="65" t="n"/>
+      <c r="V171" s="57" t="n"/>
+      <c r="W171" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X171" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y171" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z171" s="43" t="n"/>
       <c r="AA171" s="43" t="n"/>
       <c r="AB171" s="43" t="n"/>
@@ -54525,32 +55110,97 @@
       <c r="IK171" s="43" t="n"/>
     </row>
     <row r="172" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A172" s="43" t="n"/>
-      <c r="C172" s="43" t="n"/>
-      <c r="D172" s="43" t="n"/>
-      <c r="E172" s="43" t="n"/>
-      <c r="F172" s="43" t="inlineStr">
+      <c r="A172" s="48" t="n">
+        <v>170</v>
+      </c>
+      <c r="B172" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C172" s="50" t="n"/>
+      <c r="D172" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E172" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F172" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G172" s="43" t="n"/>
-      <c r="H172" s="43" t="n"/>
-      <c r="I172" s="43" t="n"/>
-      <c r="J172" s="43" t="n"/>
-      <c r="K172" s="43" t="n"/>
-      <c r="L172" s="43" t="n"/>
-      <c r="O172" s="43" t="n"/>
-      <c r="P172" s="43" t="n"/>
-      <c r="Q172" s="43" t="n"/>
-      <c r="R172" s="43" t="n"/>
-      <c r="S172" s="43" t="n"/>
-      <c r="T172" s="43" t="n"/>
-      <c r="U172" s="43" t="n"/>
-      <c r="V172" s="43" t="n"/>
-      <c r="W172" s="43" t="n"/>
-      <c r="X172" s="43" t="n"/>
-      <c r="Y172" s="43" t="n"/>
+      <c r="G172" s="49" t="n"/>
+      <c r="H172" s="51" t="inlineStr">
+        <is>
+          <t>Koura</t>
+        </is>
+      </c>
+      <c r="I172" s="51" t="inlineStr">
+        <is>
+          <t>Tangara</t>
+        </is>
+      </c>
+      <c r="J172" s="51" t="inlineStr">
+        <is>
+          <t>Koura Tangara</t>
+        </is>
+      </c>
+      <c r="K172" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L172" s="53" t="inlineStr">
+        <is>
+          <t>DIABETOLOGIST</t>
+        </is>
+      </c>
+      <c r="M172" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N172" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O172" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P172" s="51" t="inlineStr">
+        <is>
+          <t>Csref I</t>
+        </is>
+      </c>
+      <c r="Q172" s="54" t="n"/>
+      <c r="R172" s="55" t="inlineStr">
+        <is>
+          <t>66792478</t>
+        </is>
+      </c>
+      <c r="S172" s="55" t="n"/>
+      <c r="T172" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U172" s="65" t="n"/>
+      <c r="V172" s="57" t="n"/>
+      <c r="W172" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X172" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y172" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z172" s="43" t="n"/>
       <c r="AA172" s="43" t="n"/>
       <c r="AB172" s="43" t="n"/>
@@ -54773,32 +55423,97 @@
       <c r="IK172" s="43" t="n"/>
     </row>
     <row r="173" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A173" s="43" t="n"/>
-      <c r="C173" s="43" t="n"/>
-      <c r="D173" s="43" t="n"/>
-      <c r="E173" s="43" t="n"/>
-      <c r="F173" s="43" t="inlineStr">
+      <c r="A173" s="48" t="n">
+        <v>171</v>
+      </c>
+      <c r="B173" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C173" s="50" t="n"/>
+      <c r="D173" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E173" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F173" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G173" s="43" t="n"/>
-      <c r="H173" s="43" t="n"/>
-      <c r="I173" s="43" t="n"/>
-      <c r="J173" s="43" t="n"/>
-      <c r="K173" s="43" t="n"/>
-      <c r="L173" s="43" t="n"/>
-      <c r="O173" s="43" t="n"/>
-      <c r="P173" s="43" t="n"/>
-      <c r="Q173" s="43" t="n"/>
-      <c r="R173" s="43" t="n"/>
-      <c r="S173" s="43" t="n"/>
-      <c r="T173" s="43" t="n"/>
-      <c r="U173" s="43" t="n"/>
-      <c r="V173" s="43" t="n"/>
-      <c r="W173" s="43" t="n"/>
-      <c r="X173" s="43" t="n"/>
-      <c r="Y173" s="43" t="n"/>
+      <c r="G173" s="49" t="n"/>
+      <c r="H173" s="51" t="inlineStr">
+        <is>
+          <t>Yohana</t>
+        </is>
+      </c>
+      <c r="I173" s="51" t="inlineStr">
+        <is>
+          <t>Coulibaly</t>
+        </is>
+      </c>
+      <c r="J173" s="51" t="inlineStr">
+        <is>
+          <t>Yohana Coulibaly</t>
+        </is>
+      </c>
+      <c r="K173" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L173" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M173" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N173" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O173" s="51" t="inlineStr">
+        <is>
+          <t>Cmad</t>
+        </is>
+      </c>
+      <c r="P173" s="51" t="inlineStr">
+        <is>
+          <t>Cmad</t>
+        </is>
+      </c>
+      <c r="Q173" s="54" t="n"/>
+      <c r="R173" s="55" t="inlineStr">
+        <is>
+          <t>66886033</t>
+        </is>
+      </c>
+      <c r="S173" s="55" t="n"/>
+      <c r="T173" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U173" s="65" t="n"/>
+      <c r="V173" s="57" t="n"/>
+      <c r="W173" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X173" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y173" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z173" s="43" t="n"/>
       <c r="AA173" s="43" t="n"/>
       <c r="AB173" s="43" t="n"/>
@@ -55021,32 +55736,97 @@
       <c r="IK173" s="43" t="n"/>
     </row>
     <row r="174" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A174" s="43" t="n"/>
-      <c r="C174" s="43" t="n"/>
-      <c r="D174" s="43" t="n"/>
-      <c r="E174" s="43" t="n"/>
-      <c r="F174" s="43" t="inlineStr">
+      <c r="A174" s="48" t="n">
+        <v>172</v>
+      </c>
+      <c r="B174" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C174" s="50" t="n"/>
+      <c r="D174" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E174" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F174" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G174" s="43" t="n"/>
-      <c r="H174" s="43" t="n"/>
-      <c r="I174" s="43" t="n"/>
-      <c r="J174" s="43" t="n"/>
-      <c r="K174" s="43" t="n"/>
-      <c r="L174" s="43" t="n"/>
-      <c r="O174" s="43" t="n"/>
-      <c r="P174" s="43" t="n"/>
-      <c r="Q174" s="43" t="n"/>
-      <c r="R174" s="43" t="n"/>
-      <c r="S174" s="43" t="n"/>
-      <c r="T174" s="43" t="n"/>
-      <c r="U174" s="43" t="n"/>
-      <c r="V174" s="43" t="n"/>
-      <c r="W174" s="43" t="n"/>
-      <c r="X174" s="43" t="n"/>
-      <c r="Y174" s="43" t="n"/>
+      <c r="G174" s="49" t="n"/>
+      <c r="H174" s="51" t="inlineStr">
+        <is>
+          <t>Karim</t>
+        </is>
+      </c>
+      <c r="I174" s="51" t="inlineStr">
+        <is>
+          <t>Fomba</t>
+        </is>
+      </c>
+      <c r="J174" s="51" t="inlineStr">
+        <is>
+          <t>Karim Fomba</t>
+        </is>
+      </c>
+      <c r="K174" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L174" s="53" t="inlineStr">
+        <is>
+          <t>CONSULTANT PHYSICIAN</t>
+        </is>
+      </c>
+      <c r="M174" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N174" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O174" s="51" t="inlineStr">
+        <is>
+          <t>Asacoboul2</t>
+        </is>
+      </c>
+      <c r="P174" s="51" t="inlineStr">
+        <is>
+          <t>Asacoboul2</t>
+        </is>
+      </c>
+      <c r="Q174" s="54" t="n"/>
+      <c r="R174" s="55" t="inlineStr">
+        <is>
+          <t>66712575</t>
+        </is>
+      </c>
+      <c r="S174" s="55" t="n"/>
+      <c r="T174" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U174" s="65" t="n"/>
+      <c r="V174" s="57" t="n"/>
+      <c r="W174" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X174" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y174" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z174" s="43" t="n"/>
       <c r="AA174" s="43" t="n"/>
       <c r="AB174" s="43" t="n"/>
@@ -55269,32 +56049,97 @@
       <c r="IK174" s="43" t="n"/>
     </row>
     <row r="175" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A175" s="43" t="n"/>
-      <c r="C175" s="43" t="n"/>
-      <c r="D175" s="43" t="n"/>
-      <c r="E175" s="43" t="n"/>
-      <c r="F175" s="43" t="inlineStr">
+      <c r="A175" s="48" t="n">
+        <v>173</v>
+      </c>
+      <c r="B175" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C175" s="50" t="n"/>
+      <c r="D175" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E175" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F175" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G175" s="43" t="n"/>
-      <c r="H175" s="43" t="n"/>
-      <c r="I175" s="43" t="n"/>
-      <c r="J175" s="43" t="n"/>
-      <c r="K175" s="43" t="n"/>
-      <c r="L175" s="43" t="n"/>
-      <c r="O175" s="43" t="n"/>
-      <c r="P175" s="43" t="n"/>
-      <c r="Q175" s="43" t="n"/>
-      <c r="R175" s="43" t="n"/>
-      <c r="S175" s="43" t="n"/>
-      <c r="T175" s="43" t="n"/>
-      <c r="U175" s="43" t="n"/>
-      <c r="V175" s="43" t="n"/>
-      <c r="W175" s="43" t="n"/>
-      <c r="X175" s="43" t="n"/>
-      <c r="Y175" s="43" t="n"/>
+      <c r="G175" s="49" t="n"/>
+      <c r="H175" s="51" t="inlineStr">
+        <is>
+          <t>Drissa</t>
+        </is>
+      </c>
+      <c r="I175" s="51" t="inlineStr">
+        <is>
+          <t>Diarra</t>
+        </is>
+      </c>
+      <c r="J175" s="51" t="inlineStr">
+        <is>
+          <t>Drissa Diarra</t>
+        </is>
+      </c>
+      <c r="K175" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L175" s="53" t="inlineStr">
+        <is>
+          <t>DENTIST</t>
+        </is>
+      </c>
+      <c r="M175" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N175" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O175" s="51" t="inlineStr">
+        <is>
+          <t>Cherifla</t>
+        </is>
+      </c>
+      <c r="P175" s="51" t="inlineStr">
+        <is>
+          <t>Cherifla</t>
+        </is>
+      </c>
+      <c r="Q175" s="54" t="n"/>
+      <c r="R175" s="55" t="inlineStr">
+        <is>
+          <t>76332061</t>
+        </is>
+      </c>
+      <c r="S175" s="55" t="n"/>
+      <c r="T175" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U175" s="65" t="n"/>
+      <c r="V175" s="57" t="n"/>
+      <c r="W175" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X175" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y175" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z175" s="43" t="n"/>
       <c r="AA175" s="43" t="n"/>
       <c r="AB175" s="43" t="n"/>
@@ -55517,32 +56362,97 @@
       <c r="IK175" s="43" t="n"/>
     </row>
     <row r="176" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A176" s="43" t="n"/>
-      <c r="C176" s="43" t="n"/>
-      <c r="D176" s="43" t="n"/>
-      <c r="E176" s="43" t="n"/>
-      <c r="F176" s="43" t="inlineStr">
+      <c r="A176" s="48" t="n">
+        <v>174</v>
+      </c>
+      <c r="B176" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C176" s="50" t="n"/>
+      <c r="D176" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E176" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F176" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G176" s="43" t="n"/>
-      <c r="H176" s="43" t="n"/>
-      <c r="I176" s="43" t="n"/>
-      <c r="J176" s="43" t="n"/>
-      <c r="K176" s="43" t="n"/>
-      <c r="L176" s="43" t="n"/>
-      <c r="O176" s="43" t="n"/>
-      <c r="P176" s="43" t="n"/>
-      <c r="Q176" s="43" t="n"/>
-      <c r="R176" s="43" t="n"/>
-      <c r="S176" s="43" t="n"/>
-      <c r="T176" s="43" t="n"/>
-      <c r="U176" s="43" t="n"/>
-      <c r="V176" s="43" t="n"/>
-      <c r="W176" s="43" t="n"/>
-      <c r="X176" s="43" t="n"/>
-      <c r="Y176" s="43" t="n"/>
+      <c r="G176" s="49" t="n"/>
+      <c r="H176" s="51" t="inlineStr">
+        <is>
+          <t>Mamet</t>
+        </is>
+      </c>
+      <c r="I176" s="51" t="inlineStr">
+        <is>
+          <t>Sylla</t>
+        </is>
+      </c>
+      <c r="J176" s="51" t="inlineStr">
+        <is>
+          <t>Mamet Sylla</t>
+        </is>
+      </c>
+      <c r="K176" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L176" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M176" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N176" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O176" s="51" t="inlineStr">
+        <is>
+          <t>Domicile</t>
+        </is>
+      </c>
+      <c r="P176" s="51" t="inlineStr">
+        <is>
+          <t>Domicile</t>
+        </is>
+      </c>
+      <c r="Q176" s="54" t="n"/>
+      <c r="R176" s="55" t="inlineStr">
+        <is>
+          <t>66740094</t>
+        </is>
+      </c>
+      <c r="S176" s="55" t="n"/>
+      <c r="T176" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U176" s="65" t="n"/>
+      <c r="V176" s="57" t="n"/>
+      <c r="W176" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X176" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y176" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z176" s="43" t="n"/>
       <c r="AA176" s="43" t="n"/>
       <c r="AB176" s="43" t="n"/>
@@ -55765,32 +56675,97 @@
       <c r="IK176" s="43" t="n"/>
     </row>
     <row r="177" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A177" s="43" t="n"/>
-      <c r="C177" s="43" t="n"/>
-      <c r="D177" s="43" t="n"/>
-      <c r="E177" s="43" t="n"/>
-      <c r="F177" s="43" t="inlineStr">
+      <c r="A177" s="48" t="n">
+        <v>175</v>
+      </c>
+      <c r="B177" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C177" s="50" t="n"/>
+      <c r="D177" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E177" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F177" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G177" s="43" t="n"/>
-      <c r="H177" s="43" t="n"/>
-      <c r="I177" s="43" t="n"/>
-      <c r="J177" s="43" t="n"/>
-      <c r="K177" s="43" t="n"/>
-      <c r="L177" s="43" t="n"/>
-      <c r="O177" s="43" t="n"/>
-      <c r="P177" s="43" t="n"/>
-      <c r="Q177" s="43" t="n"/>
-      <c r="R177" s="43" t="n"/>
-      <c r="S177" s="43" t="n"/>
-      <c r="T177" s="43" t="n"/>
-      <c r="U177" s="43" t="n"/>
-      <c r="V177" s="43" t="n"/>
-      <c r="W177" s="43" t="n"/>
-      <c r="X177" s="43" t="n"/>
-      <c r="Y177" s="43" t="n"/>
+      <c r="G177" s="49" t="n"/>
+      <c r="H177" s="51" t="inlineStr">
+        <is>
+          <t>Ousmane</t>
+        </is>
+      </c>
+      <c r="I177" s="51" t="inlineStr">
+        <is>
+          <t>Traore</t>
+        </is>
+      </c>
+      <c r="J177" s="51" t="inlineStr">
+        <is>
+          <t>Ousmane Traore</t>
+        </is>
+      </c>
+      <c r="K177" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L177" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL SURGEON</t>
+        </is>
+      </c>
+      <c r="M177" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N177" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O177" s="51" t="inlineStr">
+        <is>
+          <t>Teriya</t>
+        </is>
+      </c>
+      <c r="P177" s="51" t="inlineStr">
+        <is>
+          <t>Teriya</t>
+        </is>
+      </c>
+      <c r="Q177" s="54" t="n"/>
+      <c r="R177" s="55" t="inlineStr">
+        <is>
+          <t>65855696</t>
+        </is>
+      </c>
+      <c r="S177" s="55" t="n"/>
+      <c r="T177" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U177" s="65" t="n"/>
+      <c r="V177" s="57" t="n"/>
+      <c r="W177" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X177" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y177" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z177" s="43" t="n"/>
       <c r="AA177" s="43" t="n"/>
       <c r="AB177" s="43" t="n"/>
@@ -56013,32 +56988,97 @@
       <c r="IK177" s="43" t="n"/>
     </row>
     <row r="178" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A178" s="43" t="n"/>
-      <c r="C178" s="43" t="n"/>
-      <c r="D178" s="43" t="n"/>
-      <c r="E178" s="43" t="n"/>
-      <c r="F178" s="43" t="inlineStr">
+      <c r="A178" s="48" t="n">
+        <v>176</v>
+      </c>
+      <c r="B178" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C178" s="50" t="n"/>
+      <c r="D178" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E178" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F178" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G178" s="43" t="n"/>
-      <c r="H178" s="43" t="n"/>
-      <c r="I178" s="43" t="n"/>
-      <c r="J178" s="43" t="n"/>
-      <c r="K178" s="43" t="n"/>
-      <c r="L178" s="43" t="n"/>
-      <c r="O178" s="43" t="n"/>
-      <c r="P178" s="43" t="n"/>
-      <c r="Q178" s="43" t="n"/>
-      <c r="R178" s="43" t="n"/>
-      <c r="S178" s="43" t="n"/>
-      <c r="T178" s="43" t="n"/>
-      <c r="U178" s="43" t="n"/>
-      <c r="V178" s="43" t="n"/>
-      <c r="W178" s="43" t="n"/>
-      <c r="X178" s="43" t="n"/>
-      <c r="Y178" s="43" t="n"/>
+      <c r="G178" s="49" t="n"/>
+      <c r="H178" s="51" t="inlineStr">
+        <is>
+          <t>Boureima</t>
+        </is>
+      </c>
+      <c r="I178" s="51" t="inlineStr">
+        <is>
+          <t>Guindob</t>
+        </is>
+      </c>
+      <c r="J178" s="51" t="inlineStr">
+        <is>
+          <t>Boureima Guindob</t>
+        </is>
+      </c>
+      <c r="K178" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L178" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL SURGEON</t>
+        </is>
+      </c>
+      <c r="M178" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N178" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O178" s="51" t="inlineStr">
+        <is>
+          <t>Sania</t>
+        </is>
+      </c>
+      <c r="P178" s="51" t="inlineStr">
+        <is>
+          <t>Sania</t>
+        </is>
+      </c>
+      <c r="Q178" s="54" t="n"/>
+      <c r="R178" s="55" t="inlineStr">
+        <is>
+          <t>65520917</t>
+        </is>
+      </c>
+      <c r="S178" s="55" t="n"/>
+      <c r="T178" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U178" s="65" t="n"/>
+      <c r="V178" s="57" t="n"/>
+      <c r="W178" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X178" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y178" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z178" s="43" t="n"/>
       <c r="AA178" s="43" t="n"/>
       <c r="AB178" s="43" t="n"/>
@@ -56261,32 +57301,97 @@
       <c r="IK178" s="43" t="n"/>
     </row>
     <row r="179" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A179" s="43" t="n"/>
-      <c r="C179" s="43" t="n"/>
-      <c r="D179" s="43" t="n"/>
-      <c r="E179" s="43" t="n"/>
-      <c r="F179" s="43" t="inlineStr">
+      <c r="A179" s="48" t="n">
+        <v>177</v>
+      </c>
+      <c r="B179" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C179" s="50" t="n"/>
+      <c r="D179" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E179" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F179" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G179" s="43" t="n"/>
-      <c r="H179" s="43" t="n"/>
-      <c r="I179" s="43" t="n"/>
-      <c r="J179" s="43" t="n"/>
-      <c r="K179" s="43" t="n"/>
-      <c r="L179" s="43" t="n"/>
-      <c r="O179" s="43" t="n"/>
-      <c r="P179" s="43" t="n"/>
-      <c r="Q179" s="43" t="n"/>
-      <c r="R179" s="43" t="n"/>
-      <c r="S179" s="43" t="n"/>
-      <c r="T179" s="43" t="n"/>
-      <c r="U179" s="43" t="n"/>
-      <c r="V179" s="43" t="n"/>
-      <c r="W179" s="43" t="n"/>
-      <c r="X179" s="43" t="n"/>
-      <c r="Y179" s="43" t="n"/>
+      <c r="G179" s="49" t="n"/>
+      <c r="H179" s="51" t="inlineStr">
+        <is>
+          <t>Doussou</t>
+        </is>
+      </c>
+      <c r="I179" s="51" t="inlineStr">
+        <is>
+          <t>Kouyate</t>
+        </is>
+      </c>
+      <c r="J179" s="51" t="inlineStr">
+        <is>
+          <t>Doussou Kouyate</t>
+        </is>
+      </c>
+      <c r="K179" s="52" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="L179" s="53" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="M179" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N179" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O179" s="51" t="inlineStr">
+        <is>
+          <t>Espoir</t>
+        </is>
+      </c>
+      <c r="P179" s="51" t="inlineStr">
+        <is>
+          <t>Espoir</t>
+        </is>
+      </c>
+      <c r="Q179" s="54" t="n"/>
+      <c r="R179" s="55" t="inlineStr">
+        <is>
+          <t>66909375</t>
+        </is>
+      </c>
+      <c r="S179" s="55" t="n"/>
+      <c r="T179" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U179" s="65" t="n"/>
+      <c r="V179" s="57" t="n"/>
+      <c r="W179" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X179" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y179" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z179" s="43" t="n"/>
       <c r="AA179" s="43" t="n"/>
       <c r="AB179" s="43" t="n"/>
@@ -56509,32 +57614,97 @@
       <c r="IK179" s="43" t="n"/>
     </row>
     <row r="180" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A180" s="43" t="n"/>
-      <c r="C180" s="43" t="n"/>
-      <c r="D180" s="43" t="n"/>
-      <c r="E180" s="43" t="n"/>
-      <c r="F180" s="43" t="inlineStr">
+      <c r="A180" s="48" t="n">
+        <v>178</v>
+      </c>
+      <c r="B180" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C180" s="50" t="n"/>
+      <c r="D180" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E180" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F180" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G180" s="43" t="n"/>
-      <c r="H180" s="43" t="n"/>
-      <c r="I180" s="43" t="n"/>
-      <c r="J180" s="43" t="n"/>
-      <c r="K180" s="43" t="n"/>
-      <c r="L180" s="43" t="n"/>
-      <c r="O180" s="43" t="n"/>
-      <c r="P180" s="43" t="n"/>
-      <c r="Q180" s="43" t="n"/>
-      <c r="R180" s="43" t="n"/>
-      <c r="S180" s="43" t="n"/>
-      <c r="T180" s="43" t="n"/>
-      <c r="U180" s="43" t="n"/>
-      <c r="V180" s="43" t="n"/>
-      <c r="W180" s="43" t="n"/>
-      <c r="X180" s="43" t="n"/>
-      <c r="Y180" s="43" t="n"/>
+      <c r="G180" s="49" t="n"/>
+      <c r="H180" s="51" t="inlineStr">
+        <is>
+          <t>Towa</t>
+        </is>
+      </c>
+      <c r="I180" s="51" t="inlineStr">
+        <is>
+          <t>Stephanie</t>
+        </is>
+      </c>
+      <c r="J180" s="51" t="inlineStr">
+        <is>
+          <t>Towa Stephanie</t>
+        </is>
+      </c>
+      <c r="K180" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L180" s="53" t="inlineStr">
+        <is>
+          <t>GYNECOLOGIST</t>
+        </is>
+      </c>
+      <c r="M180" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N180" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O180" s="51" t="inlineStr">
+        <is>
+          <t>CM</t>
+        </is>
+      </c>
+      <c r="P180" s="51" t="inlineStr">
+        <is>
+          <t>CM EPHRATA</t>
+        </is>
+      </c>
+      <c r="Q180" s="54" t="n"/>
+      <c r="R180" s="55" t="inlineStr">
+        <is>
+          <t>76432702</t>
+        </is>
+      </c>
+      <c r="S180" s="55" t="n"/>
+      <c r="T180" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U180" s="65" t="n"/>
+      <c r="V180" s="57" t="n"/>
+      <c r="W180" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X180" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y180" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z180" s="43" t="n"/>
       <c r="AA180" s="43" t="n"/>
       <c r="AB180" s="43" t="n"/>
@@ -56757,32 +57927,97 @@
       <c r="IK180" s="43" t="n"/>
     </row>
     <row r="181" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A181" s="43" t="n"/>
-      <c r="C181" s="43" t="n"/>
-      <c r="D181" s="43" t="n"/>
-      <c r="E181" s="43" t="n"/>
-      <c r="F181" s="43" t="inlineStr">
+      <c r="A181" s="48" t="n">
+        <v>179</v>
+      </c>
+      <c r="B181" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C181" s="50" t="n"/>
+      <c r="D181" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E181" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F181" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G181" s="43" t="n"/>
-      <c r="H181" s="43" t="n"/>
-      <c r="I181" s="43" t="n"/>
-      <c r="J181" s="43" t="n"/>
-      <c r="K181" s="43" t="n"/>
-      <c r="L181" s="43" t="n"/>
-      <c r="O181" s="43" t="n"/>
-      <c r="P181" s="43" t="n"/>
-      <c r="Q181" s="43" t="n"/>
-      <c r="R181" s="43" t="n"/>
-      <c r="S181" s="43" t="n"/>
-      <c r="T181" s="43" t="n"/>
-      <c r="U181" s="43" t="n"/>
-      <c r="V181" s="43" t="n"/>
-      <c r="W181" s="43" t="n"/>
-      <c r="X181" s="43" t="n"/>
-      <c r="Y181" s="43" t="n"/>
+      <c r="G181" s="49" t="n"/>
+      <c r="H181" s="51" t="inlineStr">
+        <is>
+          <t>Mamadou</t>
+        </is>
+      </c>
+      <c r="I181" s="51" t="inlineStr">
+        <is>
+          <t>Simpara</t>
+        </is>
+      </c>
+      <c r="J181" s="51" t="inlineStr">
+        <is>
+          <t>Mamadou Simpara</t>
+        </is>
+      </c>
+      <c r="K181" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L181" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M181" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N181" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O181" s="51" t="inlineStr">
+        <is>
+          <t>Teriya</t>
+        </is>
+      </c>
+      <c r="P181" s="51" t="inlineStr">
+        <is>
+          <t>Teriya</t>
+        </is>
+      </c>
+      <c r="Q181" s="54" t="n"/>
+      <c r="R181" s="55" t="inlineStr">
+        <is>
+          <t>66727852</t>
+        </is>
+      </c>
+      <c r="S181" s="55" t="n"/>
+      <c r="T181" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U181" s="65" t="n"/>
+      <c r="V181" s="57" t="n"/>
+      <c r="W181" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X181" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y181" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z181" s="43" t="n"/>
       <c r="AA181" s="43" t="n"/>
       <c r="AB181" s="43" t="n"/>
@@ -57005,32 +58240,97 @@
       <c r="IK181" s="43" t="n"/>
     </row>
     <row r="182" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A182" s="43" t="n"/>
-      <c r="C182" s="43" t="n"/>
-      <c r="D182" s="43" t="n"/>
-      <c r="E182" s="43" t="n"/>
-      <c r="F182" s="43" t="inlineStr">
+      <c r="A182" s="48" t="n">
+        <v>180</v>
+      </c>
+      <c r="B182" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C182" s="50" t="n"/>
+      <c r="D182" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E182" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F182" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G182" s="43" t="n"/>
-      <c r="H182" s="43" t="n"/>
-      <c r="I182" s="43" t="n"/>
-      <c r="J182" s="43" t="n"/>
-      <c r="K182" s="43" t="n"/>
-      <c r="L182" s="43" t="n"/>
-      <c r="O182" s="43" t="n"/>
-      <c r="P182" s="43" t="n"/>
-      <c r="Q182" s="43" t="n"/>
-      <c r="R182" s="43" t="n"/>
-      <c r="S182" s="43" t="n"/>
-      <c r="T182" s="43" t="n"/>
-      <c r="U182" s="43" t="n"/>
-      <c r="V182" s="43" t="n"/>
-      <c r="W182" s="43" t="n"/>
-      <c r="X182" s="43" t="n"/>
-      <c r="Y182" s="43" t="n"/>
+      <c r="G182" s="49" t="n"/>
+      <c r="H182" s="51" t="inlineStr">
+        <is>
+          <t>Djeneba</t>
+        </is>
+      </c>
+      <c r="I182" s="51" t="inlineStr">
+        <is>
+          <t>Traore</t>
+        </is>
+      </c>
+      <c r="J182" s="51" t="inlineStr">
+        <is>
+          <t>Djeneba Traore</t>
+        </is>
+      </c>
+      <c r="K182" s="52" t="inlineStr">
+        <is>
+          <t>MID WIFE</t>
+        </is>
+      </c>
+      <c r="L182" s="53" t="inlineStr">
+        <is>
+          <t>MID WIFE</t>
+        </is>
+      </c>
+      <c r="M182" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N182" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O182" s="51" t="inlineStr">
+        <is>
+          <t>Asacodje</t>
+        </is>
+      </c>
+      <c r="P182" s="51" t="inlineStr">
+        <is>
+          <t>Asacodje</t>
+        </is>
+      </c>
+      <c r="Q182" s="54" t="n"/>
+      <c r="R182" s="55" t="inlineStr">
+        <is>
+          <t>76383896</t>
+        </is>
+      </c>
+      <c r="S182" s="55" t="n"/>
+      <c r="T182" s="49" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="U182" s="65" t="n"/>
+      <c r="V182" s="57" t="n"/>
+      <c r="W182" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X182" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y182" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z182" s="43" t="n"/>
       <c r="AA182" s="43" t="n"/>
       <c r="AB182" s="43" t="n"/>
@@ -57253,32 +58553,97 @@
       <c r="IK182" s="43" t="n"/>
     </row>
     <row r="183" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A183" s="43" t="n"/>
-      <c r="C183" s="43" t="n"/>
-      <c r="D183" s="43" t="n"/>
-      <c r="E183" s="43" t="n"/>
-      <c r="F183" s="43" t="inlineStr">
+      <c r="A183" s="48" t="n">
+        <v>181</v>
+      </c>
+      <c r="B183" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C183" s="50" t="n"/>
+      <c r="D183" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E183" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F183" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G183" s="43" t="n"/>
-      <c r="H183" s="43" t="n"/>
-      <c r="I183" s="43" t="n"/>
-      <c r="J183" s="43" t="n"/>
-      <c r="K183" s="43" t="n"/>
-      <c r="L183" s="43" t="n"/>
-      <c r="O183" s="43" t="n"/>
-      <c r="P183" s="43" t="n"/>
-      <c r="Q183" s="43" t="n"/>
-      <c r="R183" s="43" t="n"/>
-      <c r="S183" s="43" t="n"/>
-      <c r="T183" s="43" t="n"/>
-      <c r="U183" s="43" t="n"/>
-      <c r="V183" s="43" t="n"/>
-      <c r="W183" s="43" t="n"/>
-      <c r="X183" s="43" t="n"/>
-      <c r="Y183" s="43" t="n"/>
+      <c r="G183" s="49" t="n"/>
+      <c r="H183" s="51" t="inlineStr">
+        <is>
+          <t>Yaya</t>
+        </is>
+      </c>
+      <c r="I183" s="51" t="inlineStr">
+        <is>
+          <t>Diarra</t>
+        </is>
+      </c>
+      <c r="J183" s="51" t="inlineStr">
+        <is>
+          <t>Yaya Diarra</t>
+        </is>
+      </c>
+      <c r="K183" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L183" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M183" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N183" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O183" s="51" t="inlineStr">
+        <is>
+          <t>Amupi</t>
+        </is>
+      </c>
+      <c r="P183" s="51" t="inlineStr">
+        <is>
+          <t>Amupi</t>
+        </is>
+      </c>
+      <c r="Q183" s="54" t="n"/>
+      <c r="R183" s="55" t="inlineStr">
+        <is>
+          <t>76139330</t>
+        </is>
+      </c>
+      <c r="S183" s="55" t="n"/>
+      <c r="T183" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U183" s="65" t="n"/>
+      <c r="V183" s="57" t="n"/>
+      <c r="W183" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X183" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y183" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z183" s="43" t="n"/>
       <c r="AA183" s="43" t="n"/>
       <c r="AB183" s="43" t="n"/>
@@ -57501,32 +58866,97 @@
       <c r="IK183" s="43" t="n"/>
     </row>
     <row r="184" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A184" s="43" t="n"/>
-      <c r="C184" s="43" t="n"/>
-      <c r="D184" s="43" t="n"/>
-      <c r="E184" s="43" t="n"/>
-      <c r="F184" s="43" t="inlineStr">
+      <c r="A184" s="48" t="n">
+        <v>182</v>
+      </c>
+      <c r="B184" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C184" s="50" t="n"/>
+      <c r="D184" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E184" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F184" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G184" s="43" t="n"/>
-      <c r="H184" s="43" t="n"/>
-      <c r="I184" s="43" t="n"/>
-      <c r="J184" s="43" t="n"/>
-      <c r="K184" s="43" t="n"/>
-      <c r="L184" s="43" t="n"/>
-      <c r="O184" s="43" t="n"/>
-      <c r="P184" s="43" t="n"/>
-      <c r="Q184" s="43" t="n"/>
-      <c r="R184" s="43" t="n"/>
-      <c r="S184" s="43" t="n"/>
-      <c r="T184" s="43" t="n"/>
-      <c r="U184" s="43" t="n"/>
-      <c r="V184" s="43" t="n"/>
-      <c r="W184" s="43" t="n"/>
-      <c r="X184" s="43" t="n"/>
-      <c r="Y184" s="43" t="n"/>
+      <c r="G184" s="49" t="n"/>
+      <c r="H184" s="51" t="inlineStr">
+        <is>
+          <t>Youssouf</t>
+        </is>
+      </c>
+      <c r="I184" s="51" t="inlineStr">
+        <is>
+          <t>Diakite</t>
+        </is>
+      </c>
+      <c r="J184" s="51" t="inlineStr">
+        <is>
+          <t>Youssouf Diakite</t>
+        </is>
+      </c>
+      <c r="K184" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L184" s="53" t="inlineStr">
+        <is>
+          <t>DIABETOLOGIST</t>
+        </is>
+      </c>
+      <c r="M184" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N184" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O184" s="51" t="inlineStr">
+        <is>
+          <t>Groupe</t>
+        </is>
+      </c>
+      <c r="P184" s="51" t="inlineStr">
+        <is>
+          <t>Groupe Medical</t>
+        </is>
+      </c>
+      <c r="Q184" s="54" t="n"/>
+      <c r="R184" s="55" t="inlineStr">
+        <is>
+          <t>76935493</t>
+        </is>
+      </c>
+      <c r="S184" s="55" t="n"/>
+      <c r="T184" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U184" s="65" t="n"/>
+      <c r="V184" s="57" t="n"/>
+      <c r="W184" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X184" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y184" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z184" s="43" t="n"/>
       <c r="AA184" s="43" t="n"/>
       <c r="AB184" s="43" t="n"/>
@@ -57749,32 +59179,97 @@
       <c r="IK184" s="43" t="n"/>
     </row>
     <row r="185" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A185" s="43" t="n"/>
-      <c r="C185" s="43" t="n"/>
-      <c r="D185" s="43" t="n"/>
-      <c r="E185" s="43" t="n"/>
-      <c r="F185" s="43" t="inlineStr">
+      <c r="A185" s="48" t="n">
+        <v>183</v>
+      </c>
+      <c r="B185" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C185" s="50" t="n"/>
+      <c r="D185" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E185" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F185" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G185" s="43" t="n"/>
-      <c r="H185" s="43" t="n"/>
-      <c r="I185" s="43" t="n"/>
-      <c r="J185" s="43" t="n"/>
-      <c r="K185" s="43" t="n"/>
-      <c r="L185" s="43" t="n"/>
-      <c r="O185" s="43" t="n"/>
-      <c r="P185" s="43" t="n"/>
-      <c r="Q185" s="43" t="n"/>
-      <c r="R185" s="43" t="n"/>
-      <c r="S185" s="43" t="n"/>
-      <c r="T185" s="43" t="n"/>
-      <c r="U185" s="43" t="n"/>
-      <c r="V185" s="43" t="n"/>
-      <c r="W185" s="43" t="n"/>
-      <c r="X185" s="43" t="n"/>
-      <c r="Y185" s="43" t="n"/>
+      <c r="G185" s="49" t="n"/>
+      <c r="H185" s="51" t="inlineStr">
+        <is>
+          <t>Fatoumata</t>
+        </is>
+      </c>
+      <c r="I185" s="51" t="inlineStr">
+        <is>
+          <t>Sereme</t>
+        </is>
+      </c>
+      <c r="J185" s="51" t="inlineStr">
+        <is>
+          <t>Fatoumata Sereme</t>
+        </is>
+      </c>
+      <c r="K185" s="52" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="L185" s="53" t="inlineStr">
+        <is>
+          <t>NURSE</t>
+        </is>
+      </c>
+      <c r="M185" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N185" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O185" s="51" t="inlineStr">
+        <is>
+          <t>Asacoba</t>
+        </is>
+      </c>
+      <c r="P185" s="51" t="inlineStr">
+        <is>
+          <t>Asacoba</t>
+        </is>
+      </c>
+      <c r="Q185" s="54" t="n"/>
+      <c r="R185" s="55" t="inlineStr">
+        <is>
+          <t>82432295</t>
+        </is>
+      </c>
+      <c r="S185" s="55" t="n"/>
+      <c r="T185" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U185" s="65" t="n"/>
+      <c r="V185" s="57" t="n"/>
+      <c r="W185" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X185" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y185" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z185" s="43" t="n"/>
       <c r="AA185" s="43" t="n"/>
       <c r="AB185" s="43" t="n"/>
@@ -57997,32 +59492,97 @@
       <c r="IK185" s="43" t="n"/>
     </row>
     <row r="186" ht="12.5" customFormat="1" customHeight="1" s="58">
-      <c r="A186" s="43" t="n"/>
-      <c r="C186" s="43" t="n"/>
-      <c r="D186" s="43" t="n"/>
-      <c r="E186" s="43" t="n"/>
-      <c r="F186" s="43" t="inlineStr">
+      <c r="A186" s="48" t="n">
+        <v>184</v>
+      </c>
+      <c r="B186" s="49" t="inlineStr">
+        <is>
+          <t>MALI</t>
+        </is>
+      </c>
+      <c r="C186" s="50" t="n"/>
+      <c r="D186" s="50" t="inlineStr">
+        <is>
+          <t>Alpha Kebe</t>
+        </is>
+      </c>
+      <c r="E186" s="49" t="inlineStr">
+        <is>
+          <t>Bamako</t>
+        </is>
+      </c>
+      <c r="F186" s="49" t="inlineStr">
         <is>
           <t>Team 1</t>
         </is>
       </c>
-      <c r="G186" s="43" t="n"/>
-      <c r="H186" s="43" t="n"/>
-      <c r="I186" s="43" t="n"/>
-      <c r="J186" s="43" t="n"/>
-      <c r="K186" s="43" t="n"/>
-      <c r="L186" s="43" t="n"/>
-      <c r="O186" s="43" t="n"/>
-      <c r="P186" s="43" t="n"/>
-      <c r="Q186" s="43" t="n"/>
-      <c r="R186" s="43" t="n"/>
-      <c r="S186" s="43" t="n"/>
-      <c r="T186" s="43" t="n"/>
-      <c r="U186" s="43" t="n"/>
-      <c r="V186" s="43" t="n"/>
-      <c r="W186" s="43" t="n"/>
-      <c r="X186" s="43" t="n"/>
-      <c r="Y186" s="43" t="n"/>
+      <c r="G186" s="49" t="n"/>
+      <c r="H186" s="51" t="inlineStr">
+        <is>
+          <t>Mamadou</t>
+        </is>
+      </c>
+      <c r="I186" s="51" t="inlineStr">
+        <is>
+          <t>Banou</t>
+        </is>
+      </c>
+      <c r="J186" s="51" t="inlineStr">
+        <is>
+          <t>Mamadou Banou</t>
+        </is>
+      </c>
+      <c r="K186" s="52" t="inlineStr">
+        <is>
+          <t>MEDICINE</t>
+        </is>
+      </c>
+      <c r="L186" s="53" t="inlineStr">
+        <is>
+          <t>GENERAL PRACTITIONER</t>
+        </is>
+      </c>
+      <c r="M186" s="51" t="n">
+        <v>3</v>
+      </c>
+      <c r="N186" s="51" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="O186" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="P186" s="51" t="inlineStr">
+        <is>
+          <t>Csref</t>
+        </is>
+      </c>
+      <c r="Q186" s="54" t="n"/>
+      <c r="R186" s="55" t="inlineStr">
+        <is>
+          <t>77978115</t>
+        </is>
+      </c>
+      <c r="S186" s="55" t="n"/>
+      <c r="T186" s="49" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U186" s="65" t="n"/>
+      <c r="V186" s="57" t="n"/>
+      <c r="W186" s="54" t="n">
+        <v>660000</v>
+      </c>
+      <c r="X186" s="54" t="n">
+        <v>132000</v>
+      </c>
+      <c r="Y186" s="54" t="n">
+        <v>10</v>
+      </c>
       <c r="Z186" s="43" t="n"/>
       <c r="AA186" s="43" t="n"/>
       <c r="AB186" s="43" t="n"/>

</xml_diff>

<commit_message>
BUS TO DIV: passer de 20% à 8% du TOTAL_POTENTIAL
- CORE: 660000 x 8% = 52800 (99 lignes)
- NON CORE: 330000 x 8% = 26400 (85 lignes)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alpha_Kebe liste des prescripteur.xlsx
+++ b/Alpha_Kebe liste des prescripteur.xlsx
@@ -2579,7 +2579,7 @@
         <v>330000</v>
       </c>
       <c r="X3" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y3" s="54" t="n">
         <v>5</v>
@@ -2668,7 +2668,7 @@
         <v>330000</v>
       </c>
       <c r="X4" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y4" s="54" t="n">
         <v>5</v>
@@ -2977,7 +2977,7 @@
         <v>330000</v>
       </c>
       <c r="X5" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y5" s="54" t="n">
         <v>5</v>
@@ -3286,7 +3286,7 @@
         <v>330000</v>
       </c>
       <c r="X6" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y6" s="54" t="n">
         <v>5</v>
@@ -3595,7 +3595,7 @@
         <v>660000</v>
       </c>
       <c r="X7" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y7" s="54" t="n">
         <v>10</v>
@@ -3904,7 +3904,7 @@
         <v>660000</v>
       </c>
       <c r="X8" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y8" s="54" t="n">
         <v>10</v>
@@ -4213,7 +4213,7 @@
         <v>330000</v>
       </c>
       <c r="X9" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y9" s="54" t="n">
         <v>5</v>
@@ -4522,7 +4522,7 @@
         <v>330000</v>
       </c>
       <c r="X10" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y10" s="54" t="n">
         <v>5</v>
@@ -4831,7 +4831,7 @@
         <v>330000</v>
       </c>
       <c r="X11" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y11" s="54" t="n">
         <v>5</v>
@@ -5140,7 +5140,7 @@
         <v>660000</v>
       </c>
       <c r="X12" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y12" s="54" t="n">
         <v>10</v>
@@ -5449,7 +5449,7 @@
         <v>660000</v>
       </c>
       <c r="X13" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y13" s="54" t="n">
         <v>10</v>
@@ -5758,7 +5758,7 @@
         <v>660000</v>
       </c>
       <c r="X14" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y14" s="54" t="n">
         <v>10</v>
@@ -6067,7 +6067,7 @@
         <v>660000</v>
       </c>
       <c r="X15" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y15" s="54" t="n">
         <v>10</v>
@@ -6376,7 +6376,7 @@
         <v>660000</v>
       </c>
       <c r="X16" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y16" s="54" t="n">
         <v>10</v>
@@ -6685,7 +6685,7 @@
         <v>330000</v>
       </c>
       <c r="X17" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y17" s="54" t="n">
         <v>5</v>
@@ -6993,7 +6993,7 @@
         <v>330000</v>
       </c>
       <c r="X18" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y18" s="54" t="n">
         <v>5</v>
@@ -7302,7 +7302,7 @@
         <v>660000</v>
       </c>
       <c r="X19" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y19" s="54" t="n">
         <v>10</v>
@@ -7611,7 +7611,7 @@
         <v>660000</v>
       </c>
       <c r="X20" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y20" s="54" t="n">
         <v>10</v>
@@ -7920,7 +7920,7 @@
         <v>660000</v>
       </c>
       <c r="X21" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y21" s="54" t="n">
         <v>10</v>
@@ -8229,7 +8229,7 @@
         <v>660000</v>
       </c>
       <c r="X22" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y22" s="54" t="n">
         <v>10</v>
@@ -8538,7 +8538,7 @@
         <v>660000</v>
       </c>
       <c r="X23" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y23" s="54" t="n">
         <v>10</v>
@@ -8846,7 +8846,7 @@
         <v>660000</v>
       </c>
       <c r="X24" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y24" s="54" t="n">
         <v>10</v>
@@ -9154,7 +9154,7 @@
         <v>660000</v>
       </c>
       <c r="X25" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y25" s="54" t="n">
         <v>10</v>
@@ -9462,7 +9462,7 @@
         <v>330000</v>
       </c>
       <c r="X26" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y26" s="54" t="n">
         <v>5</v>
@@ -9770,7 +9770,7 @@
         <v>660000</v>
       </c>
       <c r="X27" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y27" s="54" t="n">
         <v>10</v>
@@ -10078,7 +10078,7 @@
         <v>660000</v>
       </c>
       <c r="X28" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y28" s="54" t="n">
         <v>10</v>
@@ -10386,7 +10386,7 @@
         <v>330000</v>
       </c>
       <c r="X29" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y29" s="54" t="n">
         <v>5</v>
@@ -10694,7 +10694,7 @@
         <v>330000</v>
       </c>
       <c r="X30" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y30" s="54" t="n">
         <v>5</v>
@@ -11002,7 +11002,7 @@
         <v>330000</v>
       </c>
       <c r="X31" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y31" s="54" t="n">
         <v>5</v>
@@ -11310,7 +11310,7 @@
         <v>330000</v>
       </c>
       <c r="X32" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y32" s="54" t="n">
         <v>5</v>
@@ -11618,7 +11618,7 @@
         <v>660000</v>
       </c>
       <c r="X33" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y33" s="54" t="n">
         <v>10</v>
@@ -11926,7 +11926,7 @@
         <v>660000</v>
       </c>
       <c r="X34" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y34" s="54" t="n">
         <v>10</v>
@@ -12234,7 +12234,7 @@
         <v>660000</v>
       </c>
       <c r="X35" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y35" s="54" t="n">
         <v>10</v>
@@ -12542,7 +12542,7 @@
         <v>660000</v>
       </c>
       <c r="X36" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y36" s="54" t="n">
         <v>10</v>
@@ -12850,7 +12850,7 @@
         <v>660000</v>
       </c>
       <c r="X37" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y37" s="54" t="n">
         <v>10</v>
@@ -13158,7 +13158,7 @@
         <v>330000</v>
       </c>
       <c r="X38" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y38" s="54" t="n">
         <v>5</v>
@@ -13466,7 +13466,7 @@
         <v>660000</v>
       </c>
       <c r="X39" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y39" s="54" t="n">
         <v>10</v>
@@ -13774,7 +13774,7 @@
         <v>660000</v>
       </c>
       <c r="X40" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y40" s="54" t="n">
         <v>10</v>
@@ -14082,7 +14082,7 @@
         <v>660000</v>
       </c>
       <c r="X41" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y41" s="54" t="n">
         <v>10</v>
@@ -14390,7 +14390,7 @@
         <v>660000</v>
       </c>
       <c r="X42" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y42" s="54" t="n">
         <v>10</v>
@@ -14698,7 +14698,7 @@
         <v>660000</v>
       </c>
       <c r="X43" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y43" s="54" t="n">
         <v>10</v>
@@ -15006,7 +15006,7 @@
         <v>330000</v>
       </c>
       <c r="X44" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y44" s="54" t="n">
         <v>5</v>
@@ -15314,7 +15314,7 @@
         <v>660000</v>
       </c>
       <c r="X45" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y45" s="54" t="n">
         <v>10</v>
@@ -15622,7 +15622,7 @@
         <v>660000</v>
       </c>
       <c r="X46" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y46" s="54" t="n">
         <v>10</v>
@@ -15930,7 +15930,7 @@
         <v>330000</v>
       </c>
       <c r="X47" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y47" s="54" t="n">
         <v>5</v>
@@ -16238,7 +16238,7 @@
         <v>330000</v>
       </c>
       <c r="X48" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y48" s="54" t="n">
         <v>5</v>
@@ -16546,7 +16546,7 @@
         <v>330000</v>
       </c>
       <c r="X49" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y49" s="54" t="n">
         <v>5</v>
@@ -16854,7 +16854,7 @@
         <v>330000</v>
       </c>
       <c r="X50" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y50" s="54" t="n">
         <v>5</v>
@@ -17162,7 +17162,7 @@
         <v>330000</v>
       </c>
       <c r="X51" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y51" s="54" t="n">
         <v>5</v>
@@ -17470,7 +17470,7 @@
         <v>330000</v>
       </c>
       <c r="X52" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y52" s="54" t="n">
         <v>5</v>
@@ -17778,7 +17778,7 @@
         <v>330000</v>
       </c>
       <c r="X53" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y53" s="54" t="n">
         <v>5</v>
@@ -18086,7 +18086,7 @@
         <v>330000</v>
       </c>
       <c r="X54" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y54" s="54" t="n">
         <v>5</v>
@@ -18394,7 +18394,7 @@
         <v>330000</v>
       </c>
       <c r="X55" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y55" s="54" t="n">
         <v>5</v>
@@ -18702,7 +18702,7 @@
         <v>330000</v>
       </c>
       <c r="X56" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y56" s="54" t="n">
         <v>5</v>
@@ -19010,7 +19010,7 @@
         <v>330000</v>
       </c>
       <c r="X57" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y57" s="54" t="n">
         <v>5</v>
@@ -19318,7 +19318,7 @@
         <v>330000</v>
       </c>
       <c r="X58" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y58" s="54" t="n">
         <v>5</v>
@@ -19626,7 +19626,7 @@
         <v>330000</v>
       </c>
       <c r="X59" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y59" s="54" t="n">
         <v>5</v>
@@ -19934,7 +19934,7 @@
         <v>660000</v>
       </c>
       <c r="X60" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y60" s="54" t="n">
         <v>10</v>
@@ -20242,7 +20242,7 @@
         <v>660000</v>
       </c>
       <c r="X61" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y61" s="54" t="n">
         <v>10</v>
@@ -20550,7 +20550,7 @@
         <v>660000</v>
       </c>
       <c r="X62" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y62" s="54" t="n">
         <v>10</v>
@@ -20858,7 +20858,7 @@
         <v>330000</v>
       </c>
       <c r="X63" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y63" s="54" t="n">
         <v>5</v>
@@ -21166,7 +21166,7 @@
         <v>330000</v>
       </c>
       <c r="X64" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y64" s="54" t="n">
         <v>5</v>
@@ -21474,7 +21474,7 @@
         <v>330000</v>
       </c>
       <c r="X65" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y65" s="54" t="n">
         <v>5</v>
@@ -21782,7 +21782,7 @@
         <v>660000</v>
       </c>
       <c r="X66" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y66" s="54" t="n">
         <v>10</v>
@@ -22090,7 +22090,7 @@
         <v>330000</v>
       </c>
       <c r="X67" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y67" s="54" t="n">
         <v>5</v>
@@ -22398,7 +22398,7 @@
         <v>330000</v>
       </c>
       <c r="X68" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y68" s="54" t="n">
         <v>5</v>
@@ -22706,7 +22706,7 @@
         <v>330000</v>
       </c>
       <c r="X69" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y69" s="54" t="n">
         <v>5</v>
@@ -23014,7 +23014,7 @@
         <v>330000</v>
       </c>
       <c r="X70" s="43" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y70" s="54" t="n">
         <v>5</v>
@@ -23322,7 +23322,7 @@
         <v>660000</v>
       </c>
       <c r="X71" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y71" s="54" t="n">
         <v>10</v>
@@ -23630,7 +23630,7 @@
         <v>660000</v>
       </c>
       <c r="X72" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y72" s="54" t="n">
         <v>10</v>
@@ -23938,7 +23938,7 @@
         <v>660000</v>
       </c>
       <c r="X73" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y73" s="54" t="n">
         <v>10</v>
@@ -24247,7 +24247,7 @@
         <v>660000</v>
       </c>
       <c r="X74" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y74" s="54" t="n">
         <v>10</v>
@@ -24555,7 +24555,7 @@
         <v>660000</v>
       </c>
       <c r="X75" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y75" s="54" t="n">
         <v>10</v>
@@ -24863,7 +24863,7 @@
         <v>660000</v>
       </c>
       <c r="X76" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y76" s="54" t="n">
         <v>10</v>
@@ -25171,7 +25171,7 @@
         <v>660000</v>
       </c>
       <c r="X77" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y77" s="54" t="n">
         <v>10</v>
@@ -25479,7 +25479,7 @@
         <v>660000</v>
       </c>
       <c r="X78" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y78" s="54" t="n">
         <v>10</v>
@@ -25787,7 +25787,7 @@
         <v>660000</v>
       </c>
       <c r="X79" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y79" s="54" t="n">
         <v>10</v>
@@ -26095,7 +26095,7 @@
         <v>660000</v>
       </c>
       <c r="X80" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y80" s="54" t="n">
         <v>10</v>
@@ -26403,7 +26403,7 @@
         <v>660000</v>
       </c>
       <c r="X81" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y81" s="54" t="n">
         <v>10</v>
@@ -26711,7 +26711,7 @@
         <v>660000</v>
       </c>
       <c r="X82" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y82" s="54" t="n">
         <v>10</v>
@@ -27019,7 +27019,7 @@
         <v>660000</v>
       </c>
       <c r="X83" s="43" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y83" s="54" t="n">
         <v>10</v>
@@ -27327,7 +27327,7 @@
         <v>660000</v>
       </c>
       <c r="X84" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y84" s="54" t="n">
         <v>10</v>
@@ -27635,7 +27635,7 @@
         <v>660000</v>
       </c>
       <c r="X85" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y85" s="54" t="n">
         <v>10</v>
@@ -27943,7 +27943,7 @@
         <v>660000</v>
       </c>
       <c r="X86" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y86" s="54" t="n">
         <v>10</v>
@@ -28251,7 +28251,7 @@
         <v>330000</v>
       </c>
       <c r="X87" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y87" s="54" t="n">
         <v>5</v>
@@ -28559,7 +28559,7 @@
         <v>330000</v>
       </c>
       <c r="X88" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y88" s="54" t="n">
         <v>5</v>
@@ -28868,7 +28868,7 @@
         <v>660000</v>
       </c>
       <c r="X89" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y89" s="54" t="n">
         <v>10</v>
@@ -29177,7 +29177,7 @@
         <v>660000</v>
       </c>
       <c r="X90" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y90" s="54" t="n">
         <v>10</v>
@@ -29486,7 +29486,7 @@
         <v>330000</v>
       </c>
       <c r="X91" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y91" s="54" t="n">
         <v>5</v>
@@ -29795,7 +29795,7 @@
         <v>660000</v>
       </c>
       <c r="X92" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y92" s="54" t="n">
         <v>10</v>
@@ -30104,7 +30104,7 @@
         <v>330000</v>
       </c>
       <c r="X93" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y93" s="54" t="n">
         <v>5</v>
@@ -30413,7 +30413,7 @@
         <v>660000</v>
       </c>
       <c r="X94" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y94" s="54" t="n">
         <v>10</v>
@@ -30722,7 +30722,7 @@
         <v>660000</v>
       </c>
       <c r="X95" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y95" s="54" t="n">
         <v>10</v>
@@ -31031,7 +31031,7 @@
         <v>330000</v>
       </c>
       <c r="X96" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y96" s="54" t="n">
         <v>5</v>
@@ -31340,7 +31340,7 @@
         <v>330000</v>
       </c>
       <c r="X97" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y97" s="54" t="n">
         <v>5</v>
@@ -31649,7 +31649,7 @@
         <v>330000</v>
       </c>
       <c r="X98" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y98" s="54" t="n">
         <v>5</v>
@@ -31958,7 +31958,7 @@
         <v>660000</v>
       </c>
       <c r="X99" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y99" s="54" t="n">
         <v>10</v>
@@ -32267,7 +32267,7 @@
         <v>330000</v>
       </c>
       <c r="X100" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y100" s="54" t="n">
         <v>5</v>
@@ -32576,7 +32576,7 @@
         <v>660000</v>
       </c>
       <c r="X101" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y101" s="54" t="n">
         <v>10</v>
@@ -32885,7 +32885,7 @@
         <v>330000</v>
       </c>
       <c r="X102" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y102" s="54" t="n">
         <v>5</v>
@@ -33194,7 +33194,7 @@
         <v>660000</v>
       </c>
       <c r="X103" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y103" s="54" t="n">
         <v>10</v>
@@ -33503,7 +33503,7 @@
         <v>660000</v>
       </c>
       <c r="X104" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y104" s="54" t="n">
         <v>10</v>
@@ -33812,7 +33812,7 @@
         <v>330000</v>
       </c>
       <c r="X105" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y105" s="54" t="n">
         <v>5</v>
@@ -34121,7 +34121,7 @@
         <v>330000</v>
       </c>
       <c r="X106" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y106" s="54" t="n">
         <v>5</v>
@@ -34430,7 +34430,7 @@
         <v>660000</v>
       </c>
       <c r="X107" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y107" s="54" t="n">
         <v>10</v>
@@ -34739,7 +34739,7 @@
         <v>330000</v>
       </c>
       <c r="X108" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y108" s="54" t="n">
         <v>5</v>
@@ -35048,7 +35048,7 @@
         <v>660000</v>
       </c>
       <c r="X109" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y109" s="54" t="n">
         <v>10</v>
@@ -35357,7 +35357,7 @@
         <v>660000</v>
       </c>
       <c r="X110" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y110" s="54" t="n">
         <v>10</v>
@@ -35666,7 +35666,7 @@
         <v>660000</v>
       </c>
       <c r="X111" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y111" s="54" t="n">
         <v>10</v>
@@ -35975,7 +35975,7 @@
         <v>660000</v>
       </c>
       <c r="X112" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y112" s="54" t="n">
         <v>10</v>
@@ -36284,7 +36284,7 @@
         <v>660000</v>
       </c>
       <c r="X113" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y113" s="54" t="n">
         <v>10</v>
@@ -36593,7 +36593,7 @@
         <v>660000</v>
       </c>
       <c r="X114" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y114" s="54" t="n">
         <v>10</v>
@@ -36902,7 +36902,7 @@
         <v>660000</v>
       </c>
       <c r="X115" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y115" s="54" t="n">
         <v>10</v>
@@ -37211,7 +37211,7 @@
         <v>330000</v>
       </c>
       <c r="X116" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y116" s="54" t="n">
         <v>5</v>
@@ -37520,7 +37520,7 @@
         <v>660000</v>
       </c>
       <c r="X117" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y117" s="54" t="n">
         <v>10</v>
@@ -37829,7 +37829,7 @@
         <v>660000</v>
       </c>
       <c r="X118" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y118" s="54" t="n">
         <v>10</v>
@@ -38138,7 +38138,7 @@
         <v>660000</v>
       </c>
       <c r="X119" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y119" s="54" t="n">
         <v>10</v>
@@ -38447,7 +38447,7 @@
         <v>660000</v>
       </c>
       <c r="X120" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y120" s="54" t="n">
         <v>10</v>
@@ -38756,7 +38756,7 @@
         <v>660000</v>
       </c>
       <c r="X121" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y121" s="54" t="n">
         <v>10</v>
@@ -39065,7 +39065,7 @@
         <v>660000</v>
       </c>
       <c r="X122" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y122" s="54" t="n">
         <v>10</v>
@@ -39374,7 +39374,7 @@
         <v>330000</v>
       </c>
       <c r="X123" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y123" s="54" t="n">
         <v>5</v>
@@ -39683,7 +39683,7 @@
         <v>660000</v>
       </c>
       <c r="X124" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y124" s="54" t="n">
         <v>10</v>
@@ -39992,7 +39992,7 @@
         <v>660000</v>
       </c>
       <c r="X125" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y125" s="54" t="n">
         <v>10</v>
@@ -40301,7 +40301,7 @@
         <v>660000</v>
       </c>
       <c r="X126" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y126" s="54" t="n">
         <v>10</v>
@@ -40610,7 +40610,7 @@
         <v>330000</v>
       </c>
       <c r="X127" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y127" s="54" t="n">
         <v>5</v>
@@ -40919,7 +40919,7 @@
         <v>660000</v>
       </c>
       <c r="X128" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y128" s="54" t="n">
         <v>10</v>
@@ -41228,7 +41228,7 @@
         <v>330000</v>
       </c>
       <c r="X129" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y129" s="54" t="n">
         <v>5</v>
@@ -41537,7 +41537,7 @@
         <v>330000</v>
       </c>
       <c r="X130" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y130" s="54" t="n">
         <v>5</v>
@@ -41846,7 +41846,7 @@
         <v>330000</v>
       </c>
       <c r="X131" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y131" s="54" t="n">
         <v>5</v>
@@ -42155,7 +42155,7 @@
         <v>330000</v>
       </c>
       <c r="X132" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y132" s="54" t="n">
         <v>5</v>
@@ -42464,7 +42464,7 @@
         <v>330000</v>
       </c>
       <c r="X133" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y133" s="54" t="n">
         <v>5</v>
@@ -42773,7 +42773,7 @@
         <v>330000</v>
       </c>
       <c r="X134" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y134" s="54" t="n">
         <v>5</v>
@@ -43082,7 +43082,7 @@
         <v>330000</v>
       </c>
       <c r="X135" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y135" s="54" t="n">
         <v>5</v>
@@ -43391,7 +43391,7 @@
         <v>330000</v>
       </c>
       <c r="X136" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y136" s="54" t="n">
         <v>5</v>
@@ -43700,7 +43700,7 @@
         <v>330000</v>
       </c>
       <c r="X137" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y137" s="54" t="n">
         <v>5</v>
@@ -44009,7 +44009,7 @@
         <v>330000</v>
       </c>
       <c r="X138" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y138" s="54" t="n">
         <v>5</v>
@@ -44318,7 +44318,7 @@
         <v>330000</v>
       </c>
       <c r="X139" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y139" s="54" t="n">
         <v>5</v>
@@ -44627,7 +44627,7 @@
         <v>330000</v>
       </c>
       <c r="X140" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y140" s="54" t="n">
         <v>5</v>
@@ -44936,7 +44936,7 @@
         <v>330000</v>
       </c>
       <c r="X141" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y141" s="54" t="n">
         <v>5</v>
@@ -45245,7 +45245,7 @@
         <v>330000</v>
       </c>
       <c r="X142" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y142" s="54" t="n">
         <v>5</v>
@@ -45554,7 +45554,7 @@
         <v>330000</v>
       </c>
       <c r="X143" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y143" s="54" t="n">
         <v>5</v>
@@ -45863,7 +45863,7 @@
         <v>330000</v>
       </c>
       <c r="X144" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y144" s="54" t="n">
         <v>5</v>
@@ -46172,7 +46172,7 @@
         <v>330000</v>
       </c>
       <c r="X145" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y145" s="54" t="n">
         <v>5</v>
@@ -46481,7 +46481,7 @@
         <v>330000</v>
       </c>
       <c r="X146" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y146" s="54" t="n">
         <v>5</v>
@@ -46790,7 +46790,7 @@
         <v>330000</v>
       </c>
       <c r="X147" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y147" s="54" t="n">
         <v>5</v>
@@ -47099,7 +47099,7 @@
         <v>330000</v>
       </c>
       <c r="X148" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y148" s="54" t="n">
         <v>5</v>
@@ -47408,7 +47408,7 @@
         <v>330000</v>
       </c>
       <c r="X149" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y149" s="54" t="n">
         <v>5</v>
@@ -47717,7 +47717,7 @@
         <v>330000</v>
       </c>
       <c r="X150" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y150" s="54" t="n">
         <v>5</v>
@@ -48026,7 +48026,7 @@
         <v>330000</v>
       </c>
       <c r="X151" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y151" s="54" t="n">
         <v>5</v>
@@ -48335,7 +48335,7 @@
         <v>330000</v>
       </c>
       <c r="X152" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y152" s="54" t="n">
         <v>5</v>
@@ -48644,7 +48644,7 @@
         <v>330000</v>
       </c>
       <c r="X153" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y153" s="54" t="n">
         <v>5</v>
@@ -48953,7 +48953,7 @@
         <v>330000</v>
       </c>
       <c r="X154" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y154" s="54" t="n">
         <v>5</v>
@@ -49262,7 +49262,7 @@
         <v>330000</v>
       </c>
       <c r="X155" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y155" s="54" t="n">
         <v>5</v>
@@ -49571,7 +49571,7 @@
         <v>330000</v>
       </c>
       <c r="X156" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y156" s="54" t="n">
         <v>5</v>
@@ -49880,7 +49880,7 @@
         <v>330000</v>
       </c>
       <c r="X157" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y157" s="54" t="n">
         <v>5</v>
@@ -50189,7 +50189,7 @@
         <v>330000</v>
       </c>
       <c r="X158" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y158" s="54" t="n">
         <v>5</v>
@@ -50498,7 +50498,7 @@
         <v>330000</v>
       </c>
       <c r="X159" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y159" s="54" t="n">
         <v>5</v>
@@ -50807,7 +50807,7 @@
         <v>330000</v>
       </c>
       <c r="X160" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y160" s="54" t="n">
         <v>5</v>
@@ -51116,7 +51116,7 @@
         <v>330000</v>
       </c>
       <c r="X161" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y161" s="54" t="n">
         <v>5</v>
@@ -51425,7 +51425,7 @@
         <v>330000</v>
       </c>
       <c r="X162" s="54" t="n">
-        <v>66000</v>
+        <v>26400</v>
       </c>
       <c r="Y162" s="54" t="n">
         <v>5</v>
@@ -51734,7 +51734,7 @@
         <v>660000</v>
       </c>
       <c r="X163" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y163" s="54" t="n">
         <v>10</v>
@@ -52043,7 +52043,7 @@
         <v>660000</v>
       </c>
       <c r="X164" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y164" s="54" t="n">
         <v>10</v>
@@ -52352,7 +52352,7 @@
         <v>660000</v>
       </c>
       <c r="X165" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y165" s="54" t="n">
         <v>10</v>
@@ -52661,7 +52661,7 @@
         <v>660000</v>
       </c>
       <c r="X166" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y166" s="54" t="n">
         <v>10</v>
@@ -52970,7 +52970,7 @@
         <v>660000</v>
       </c>
       <c r="X167" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y167" s="54" t="n">
         <v>10</v>
@@ -53279,7 +53279,7 @@
         <v>660000</v>
       </c>
       <c r="X168" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y168" s="54" t="n">
         <v>10</v>
@@ -53588,7 +53588,7 @@
         <v>660000</v>
       </c>
       <c r="X169" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y169" s="54" t="n">
         <v>10</v>
@@ -53897,7 +53897,7 @@
         <v>660000</v>
       </c>
       <c r="X170" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y170" s="54" t="n">
         <v>10</v>
@@ -54206,7 +54206,7 @@
         <v>660000</v>
       </c>
       <c r="X171" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y171" s="54" t="n">
         <v>10</v>
@@ -54515,7 +54515,7 @@
         <v>660000</v>
       </c>
       <c r="X172" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y172" s="54" t="n">
         <v>10</v>
@@ -54824,7 +54824,7 @@
         <v>660000</v>
       </c>
       <c r="X173" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y173" s="54" t="n">
         <v>10</v>
@@ -55133,7 +55133,7 @@
         <v>660000</v>
       </c>
       <c r="X174" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y174" s="54" t="n">
         <v>10</v>
@@ -55442,7 +55442,7 @@
         <v>660000</v>
       </c>
       <c r="X175" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y175" s="54" t="n">
         <v>10</v>
@@ -55751,7 +55751,7 @@
         <v>660000</v>
       </c>
       <c r="X176" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y176" s="54" t="n">
         <v>10</v>
@@ -56060,7 +56060,7 @@
         <v>660000</v>
       </c>
       <c r="X177" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y177" s="54" t="n">
         <v>10</v>
@@ -56369,7 +56369,7 @@
         <v>660000</v>
       </c>
       <c r="X178" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y178" s="54" t="n">
         <v>10</v>
@@ -56678,7 +56678,7 @@
         <v>660000</v>
       </c>
       <c r="X179" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y179" s="54" t="n">
         <v>10</v>
@@ -56987,7 +56987,7 @@
         <v>660000</v>
       </c>
       <c r="X180" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y180" s="54" t="n">
         <v>10</v>
@@ -57296,7 +57296,7 @@
         <v>660000</v>
       </c>
       <c r="X181" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y181" s="54" t="n">
         <v>10</v>
@@ -57605,7 +57605,7 @@
         <v>660000</v>
       </c>
       <c r="X182" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y182" s="54" t="n">
         <v>10</v>
@@ -57914,7 +57914,7 @@
         <v>660000</v>
       </c>
       <c r="X183" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y183" s="54" t="n">
         <v>10</v>
@@ -58223,7 +58223,7 @@
         <v>660000</v>
       </c>
       <c r="X184" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y184" s="54" t="n">
         <v>10</v>
@@ -58532,7 +58532,7 @@
         <v>660000</v>
       </c>
       <c r="X185" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y185" s="54" t="n">
         <v>10</v>
@@ -58841,7 +58841,7 @@
         <v>660000</v>
       </c>
       <c r="X186" s="54" t="n">
-        <v>132000</v>
+        <v>52800</v>
       </c>
       <c r="Y186" s="54" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
BUS TO DIV: passer de 8% à 5% du TOTAL_POTENTIAL
- CORE: 660000 x 5% = 33000 (99 lignes)
- NON CORE: 330000 x 5% = 16500 (85 lignes)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alpha_Kebe liste des prescripteur.xlsx
+++ b/Alpha_Kebe liste des prescripteur.xlsx
@@ -2579,7 +2579,7 @@
         <v>330000</v>
       </c>
       <c r="X3" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y3" s="54" t="n">
         <v>5</v>
@@ -2668,7 +2668,7 @@
         <v>330000</v>
       </c>
       <c r="X4" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y4" s="54" t="n">
         <v>5</v>
@@ -2977,7 +2977,7 @@
         <v>330000</v>
       </c>
       <c r="X5" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y5" s="54" t="n">
         <v>5</v>
@@ -3286,7 +3286,7 @@
         <v>330000</v>
       </c>
       <c r="X6" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y6" s="54" t="n">
         <v>5</v>
@@ -3595,7 +3595,7 @@
         <v>660000</v>
       </c>
       <c r="X7" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y7" s="54" t="n">
         <v>10</v>
@@ -3904,7 +3904,7 @@
         <v>660000</v>
       </c>
       <c r="X8" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y8" s="54" t="n">
         <v>10</v>
@@ -4213,7 +4213,7 @@
         <v>330000</v>
       </c>
       <c r="X9" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y9" s="54" t="n">
         <v>5</v>
@@ -4522,7 +4522,7 @@
         <v>330000</v>
       </c>
       <c r="X10" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y10" s="54" t="n">
         <v>5</v>
@@ -4831,7 +4831,7 @@
         <v>330000</v>
       </c>
       <c r="X11" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y11" s="54" t="n">
         <v>5</v>
@@ -5140,7 +5140,7 @@
         <v>660000</v>
       </c>
       <c r="X12" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y12" s="54" t="n">
         <v>10</v>
@@ -5449,7 +5449,7 @@
         <v>660000</v>
       </c>
       <c r="X13" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y13" s="54" t="n">
         <v>10</v>
@@ -5758,7 +5758,7 @@
         <v>660000</v>
       </c>
       <c r="X14" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y14" s="54" t="n">
         <v>10</v>
@@ -6067,7 +6067,7 @@
         <v>660000</v>
       </c>
       <c r="X15" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y15" s="54" t="n">
         <v>10</v>
@@ -6376,7 +6376,7 @@
         <v>660000</v>
       </c>
       <c r="X16" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y16" s="54" t="n">
         <v>10</v>
@@ -6685,7 +6685,7 @@
         <v>330000</v>
       </c>
       <c r="X17" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y17" s="54" t="n">
         <v>5</v>
@@ -6993,7 +6993,7 @@
         <v>330000</v>
       </c>
       <c r="X18" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y18" s="54" t="n">
         <v>5</v>
@@ -7302,7 +7302,7 @@
         <v>660000</v>
       </c>
       <c r="X19" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y19" s="54" t="n">
         <v>10</v>
@@ -7611,7 +7611,7 @@
         <v>660000</v>
       </c>
       <c r="X20" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y20" s="54" t="n">
         <v>10</v>
@@ -7920,7 +7920,7 @@
         <v>660000</v>
       </c>
       <c r="X21" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y21" s="54" t="n">
         <v>10</v>
@@ -8229,7 +8229,7 @@
         <v>660000</v>
       </c>
       <c r="X22" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y22" s="54" t="n">
         <v>10</v>
@@ -8538,7 +8538,7 @@
         <v>660000</v>
       </c>
       <c r="X23" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y23" s="54" t="n">
         <v>10</v>
@@ -8846,7 +8846,7 @@
         <v>660000</v>
       </c>
       <c r="X24" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y24" s="54" t="n">
         <v>10</v>
@@ -9154,7 +9154,7 @@
         <v>660000</v>
       </c>
       <c r="X25" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y25" s="54" t="n">
         <v>10</v>
@@ -9462,7 +9462,7 @@
         <v>330000</v>
       </c>
       <c r="X26" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y26" s="54" t="n">
         <v>5</v>
@@ -9770,7 +9770,7 @@
         <v>660000</v>
       </c>
       <c r="X27" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y27" s="54" t="n">
         <v>10</v>
@@ -10078,7 +10078,7 @@
         <v>660000</v>
       </c>
       <c r="X28" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y28" s="54" t="n">
         <v>10</v>
@@ -10386,7 +10386,7 @@
         <v>330000</v>
       </c>
       <c r="X29" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y29" s="54" t="n">
         <v>5</v>
@@ -10694,7 +10694,7 @@
         <v>330000</v>
       </c>
       <c r="X30" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y30" s="54" t="n">
         <v>5</v>
@@ -11002,7 +11002,7 @@
         <v>330000</v>
       </c>
       <c r="X31" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y31" s="54" t="n">
         <v>5</v>
@@ -11310,7 +11310,7 @@
         <v>330000</v>
       </c>
       <c r="X32" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y32" s="54" t="n">
         <v>5</v>
@@ -11618,7 +11618,7 @@
         <v>660000</v>
       </c>
       <c r="X33" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y33" s="54" t="n">
         <v>10</v>
@@ -11926,7 +11926,7 @@
         <v>660000</v>
       </c>
       <c r="X34" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y34" s="54" t="n">
         <v>10</v>
@@ -12234,7 +12234,7 @@
         <v>660000</v>
       </c>
       <c r="X35" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y35" s="54" t="n">
         <v>10</v>
@@ -12542,7 +12542,7 @@
         <v>660000</v>
       </c>
       <c r="X36" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y36" s="54" t="n">
         <v>10</v>
@@ -12850,7 +12850,7 @@
         <v>660000</v>
       </c>
       <c r="X37" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y37" s="54" t="n">
         <v>10</v>
@@ -13158,7 +13158,7 @@
         <v>330000</v>
       </c>
       <c r="X38" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y38" s="54" t="n">
         <v>5</v>
@@ -13466,7 +13466,7 @@
         <v>660000</v>
       </c>
       <c r="X39" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y39" s="54" t="n">
         <v>10</v>
@@ -13774,7 +13774,7 @@
         <v>660000</v>
       </c>
       <c r="X40" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y40" s="54" t="n">
         <v>10</v>
@@ -14082,7 +14082,7 @@
         <v>660000</v>
       </c>
       <c r="X41" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y41" s="54" t="n">
         <v>10</v>
@@ -14390,7 +14390,7 @@
         <v>660000</v>
       </c>
       <c r="X42" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y42" s="54" t="n">
         <v>10</v>
@@ -14698,7 +14698,7 @@
         <v>660000</v>
       </c>
       <c r="X43" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y43" s="54" t="n">
         <v>10</v>
@@ -15006,7 +15006,7 @@
         <v>330000</v>
       </c>
       <c r="X44" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y44" s="54" t="n">
         <v>5</v>
@@ -15314,7 +15314,7 @@
         <v>660000</v>
       </c>
       <c r="X45" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y45" s="54" t="n">
         <v>10</v>
@@ -15622,7 +15622,7 @@
         <v>660000</v>
       </c>
       <c r="X46" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y46" s="54" t="n">
         <v>10</v>
@@ -15930,7 +15930,7 @@
         <v>330000</v>
       </c>
       <c r="X47" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y47" s="54" t="n">
         <v>5</v>
@@ -16238,7 +16238,7 @@
         <v>330000</v>
       </c>
       <c r="X48" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y48" s="54" t="n">
         <v>5</v>
@@ -16546,7 +16546,7 @@
         <v>330000</v>
       </c>
       <c r="X49" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y49" s="54" t="n">
         <v>5</v>
@@ -16854,7 +16854,7 @@
         <v>330000</v>
       </c>
       <c r="X50" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y50" s="54" t="n">
         <v>5</v>
@@ -17162,7 +17162,7 @@
         <v>330000</v>
       </c>
       <c r="X51" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y51" s="54" t="n">
         <v>5</v>
@@ -17470,7 +17470,7 @@
         <v>330000</v>
       </c>
       <c r="X52" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y52" s="54" t="n">
         <v>5</v>
@@ -17778,7 +17778,7 @@
         <v>330000</v>
       </c>
       <c r="X53" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y53" s="54" t="n">
         <v>5</v>
@@ -18086,7 +18086,7 @@
         <v>330000</v>
       </c>
       <c r="X54" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y54" s="54" t="n">
         <v>5</v>
@@ -18394,7 +18394,7 @@
         <v>330000</v>
       </c>
       <c r="X55" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y55" s="54" t="n">
         <v>5</v>
@@ -18702,7 +18702,7 @@
         <v>330000</v>
       </c>
       <c r="X56" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y56" s="54" t="n">
         <v>5</v>
@@ -19010,7 +19010,7 @@
         <v>330000</v>
       </c>
       <c r="X57" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y57" s="54" t="n">
         <v>5</v>
@@ -19318,7 +19318,7 @@
         <v>330000</v>
       </c>
       <c r="X58" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y58" s="54" t="n">
         <v>5</v>
@@ -19626,7 +19626,7 @@
         <v>330000</v>
       </c>
       <c r="X59" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y59" s="54" t="n">
         <v>5</v>
@@ -19934,7 +19934,7 @@
         <v>660000</v>
       </c>
       <c r="X60" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y60" s="54" t="n">
         <v>10</v>
@@ -20242,7 +20242,7 @@
         <v>660000</v>
       </c>
       <c r="X61" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y61" s="54" t="n">
         <v>10</v>
@@ -20550,7 +20550,7 @@
         <v>660000</v>
       </c>
       <c r="X62" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y62" s="54" t="n">
         <v>10</v>
@@ -20858,7 +20858,7 @@
         <v>330000</v>
       </c>
       <c r="X63" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y63" s="54" t="n">
         <v>5</v>
@@ -21166,7 +21166,7 @@
         <v>330000</v>
       </c>
       <c r="X64" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y64" s="54" t="n">
         <v>5</v>
@@ -21474,7 +21474,7 @@
         <v>330000</v>
       </c>
       <c r="X65" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y65" s="54" t="n">
         <v>5</v>
@@ -21782,7 +21782,7 @@
         <v>660000</v>
       </c>
       <c r="X66" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y66" s="54" t="n">
         <v>10</v>
@@ -22090,7 +22090,7 @@
         <v>330000</v>
       </c>
       <c r="X67" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y67" s="54" t="n">
         <v>5</v>
@@ -22398,7 +22398,7 @@
         <v>330000</v>
       </c>
       <c r="X68" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y68" s="54" t="n">
         <v>5</v>
@@ -22706,7 +22706,7 @@
         <v>330000</v>
       </c>
       <c r="X69" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y69" s="54" t="n">
         <v>5</v>
@@ -23014,7 +23014,7 @@
         <v>330000</v>
       </c>
       <c r="X70" s="43" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y70" s="54" t="n">
         <v>5</v>
@@ -23322,7 +23322,7 @@
         <v>660000</v>
       </c>
       <c r="X71" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y71" s="54" t="n">
         <v>10</v>
@@ -23630,7 +23630,7 @@
         <v>660000</v>
       </c>
       <c r="X72" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y72" s="54" t="n">
         <v>10</v>
@@ -23938,7 +23938,7 @@
         <v>660000</v>
       </c>
       <c r="X73" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y73" s="54" t="n">
         <v>10</v>
@@ -24247,7 +24247,7 @@
         <v>660000</v>
       </c>
       <c r="X74" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y74" s="54" t="n">
         <v>10</v>
@@ -24555,7 +24555,7 @@
         <v>660000</v>
       </c>
       <c r="X75" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y75" s="54" t="n">
         <v>10</v>
@@ -24863,7 +24863,7 @@
         <v>660000</v>
       </c>
       <c r="X76" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y76" s="54" t="n">
         <v>10</v>
@@ -25171,7 +25171,7 @@
         <v>660000</v>
       </c>
       <c r="X77" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y77" s="54" t="n">
         <v>10</v>
@@ -25479,7 +25479,7 @@
         <v>660000</v>
       </c>
       <c r="X78" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y78" s="54" t="n">
         <v>10</v>
@@ -25787,7 +25787,7 @@
         <v>660000</v>
       </c>
       <c r="X79" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y79" s="54" t="n">
         <v>10</v>
@@ -26095,7 +26095,7 @@
         <v>660000</v>
       </c>
       <c r="X80" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y80" s="54" t="n">
         <v>10</v>
@@ -26403,7 +26403,7 @@
         <v>660000</v>
       </c>
       <c r="X81" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y81" s="54" t="n">
         <v>10</v>
@@ -26711,7 +26711,7 @@
         <v>660000</v>
       </c>
       <c r="X82" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y82" s="54" t="n">
         <v>10</v>
@@ -27019,7 +27019,7 @@
         <v>660000</v>
       </c>
       <c r="X83" s="43" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y83" s="54" t="n">
         <v>10</v>
@@ -27327,7 +27327,7 @@
         <v>660000</v>
       </c>
       <c r="X84" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y84" s="54" t="n">
         <v>10</v>
@@ -27635,7 +27635,7 @@
         <v>660000</v>
       </c>
       <c r="X85" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y85" s="54" t="n">
         <v>10</v>
@@ -27943,7 +27943,7 @@
         <v>660000</v>
       </c>
       <c r="X86" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y86" s="54" t="n">
         <v>10</v>
@@ -28251,7 +28251,7 @@
         <v>330000</v>
       </c>
       <c r="X87" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y87" s="54" t="n">
         <v>5</v>
@@ -28559,7 +28559,7 @@
         <v>330000</v>
       </c>
       <c r="X88" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y88" s="54" t="n">
         <v>5</v>
@@ -28868,7 +28868,7 @@
         <v>660000</v>
       </c>
       <c r="X89" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y89" s="54" t="n">
         <v>10</v>
@@ -29177,7 +29177,7 @@
         <v>660000</v>
       </c>
       <c r="X90" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y90" s="54" t="n">
         <v>10</v>
@@ -29486,7 +29486,7 @@
         <v>330000</v>
       </c>
       <c r="X91" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y91" s="54" t="n">
         <v>5</v>
@@ -29795,7 +29795,7 @@
         <v>660000</v>
       </c>
       <c r="X92" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y92" s="54" t="n">
         <v>10</v>
@@ -30104,7 +30104,7 @@
         <v>330000</v>
       </c>
       <c r="X93" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y93" s="54" t="n">
         <v>5</v>
@@ -30413,7 +30413,7 @@
         <v>660000</v>
       </c>
       <c r="X94" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y94" s="54" t="n">
         <v>10</v>
@@ -30722,7 +30722,7 @@
         <v>660000</v>
       </c>
       <c r="X95" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y95" s="54" t="n">
         <v>10</v>
@@ -31031,7 +31031,7 @@
         <v>330000</v>
       </c>
       <c r="X96" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y96" s="54" t="n">
         <v>5</v>
@@ -31340,7 +31340,7 @@
         <v>330000</v>
       </c>
       <c r="X97" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y97" s="54" t="n">
         <v>5</v>
@@ -31649,7 +31649,7 @@
         <v>330000</v>
       </c>
       <c r="X98" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y98" s="54" t="n">
         <v>5</v>
@@ -31958,7 +31958,7 @@
         <v>660000</v>
       </c>
       <c r="X99" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y99" s="54" t="n">
         <v>10</v>
@@ -32267,7 +32267,7 @@
         <v>330000</v>
       </c>
       <c r="X100" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y100" s="54" t="n">
         <v>5</v>
@@ -32576,7 +32576,7 @@
         <v>660000</v>
       </c>
       <c r="X101" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y101" s="54" t="n">
         <v>10</v>
@@ -32885,7 +32885,7 @@
         <v>330000</v>
       </c>
       <c r="X102" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y102" s="54" t="n">
         <v>5</v>
@@ -33194,7 +33194,7 @@
         <v>660000</v>
       </c>
       <c r="X103" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y103" s="54" t="n">
         <v>10</v>
@@ -33503,7 +33503,7 @@
         <v>660000</v>
       </c>
       <c r="X104" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y104" s="54" t="n">
         <v>10</v>
@@ -33812,7 +33812,7 @@
         <v>330000</v>
       </c>
       <c r="X105" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y105" s="54" t="n">
         <v>5</v>
@@ -34121,7 +34121,7 @@
         <v>330000</v>
       </c>
       <c r="X106" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y106" s="54" t="n">
         <v>5</v>
@@ -34430,7 +34430,7 @@
         <v>660000</v>
       </c>
       <c r="X107" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y107" s="54" t="n">
         <v>10</v>
@@ -34739,7 +34739,7 @@
         <v>330000</v>
       </c>
       <c r="X108" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y108" s="54" t="n">
         <v>5</v>
@@ -35048,7 +35048,7 @@
         <v>660000</v>
       </c>
       <c r="X109" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y109" s="54" t="n">
         <v>10</v>
@@ -35357,7 +35357,7 @@
         <v>660000</v>
       </c>
       <c r="X110" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y110" s="54" t="n">
         <v>10</v>
@@ -35666,7 +35666,7 @@
         <v>660000</v>
       </c>
       <c r="X111" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y111" s="54" t="n">
         <v>10</v>
@@ -35975,7 +35975,7 @@
         <v>660000</v>
       </c>
       <c r="X112" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y112" s="54" t="n">
         <v>10</v>
@@ -36284,7 +36284,7 @@
         <v>660000</v>
       </c>
       <c r="X113" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y113" s="54" t="n">
         <v>10</v>
@@ -36593,7 +36593,7 @@
         <v>660000</v>
       </c>
       <c r="X114" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y114" s="54" t="n">
         <v>10</v>
@@ -36902,7 +36902,7 @@
         <v>660000</v>
       </c>
       <c r="X115" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y115" s="54" t="n">
         <v>10</v>
@@ -37211,7 +37211,7 @@
         <v>330000</v>
       </c>
       <c r="X116" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y116" s="54" t="n">
         <v>5</v>
@@ -37520,7 +37520,7 @@
         <v>660000</v>
       </c>
       <c r="X117" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y117" s="54" t="n">
         <v>10</v>
@@ -37829,7 +37829,7 @@
         <v>660000</v>
       </c>
       <c r="X118" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y118" s="54" t="n">
         <v>10</v>
@@ -38138,7 +38138,7 @@
         <v>660000</v>
       </c>
       <c r="X119" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y119" s="54" t="n">
         <v>10</v>
@@ -38447,7 +38447,7 @@
         <v>660000</v>
       </c>
       <c r="X120" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y120" s="54" t="n">
         <v>10</v>
@@ -38756,7 +38756,7 @@
         <v>660000</v>
       </c>
       <c r="X121" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y121" s="54" t="n">
         <v>10</v>
@@ -39065,7 +39065,7 @@
         <v>660000</v>
       </c>
       <c r="X122" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y122" s="54" t="n">
         <v>10</v>
@@ -39374,7 +39374,7 @@
         <v>330000</v>
       </c>
       <c r="X123" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y123" s="54" t="n">
         <v>5</v>
@@ -39683,7 +39683,7 @@
         <v>660000</v>
       </c>
       <c r="X124" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y124" s="54" t="n">
         <v>10</v>
@@ -39992,7 +39992,7 @@
         <v>660000</v>
       </c>
       <c r="X125" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y125" s="54" t="n">
         <v>10</v>
@@ -40301,7 +40301,7 @@
         <v>660000</v>
       </c>
       <c r="X126" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y126" s="54" t="n">
         <v>10</v>
@@ -40610,7 +40610,7 @@
         <v>330000</v>
       </c>
       <c r="X127" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y127" s="54" t="n">
         <v>5</v>
@@ -40919,7 +40919,7 @@
         <v>660000</v>
       </c>
       <c r="X128" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y128" s="54" t="n">
         <v>10</v>
@@ -41228,7 +41228,7 @@
         <v>330000</v>
       </c>
       <c r="X129" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y129" s="54" t="n">
         <v>5</v>
@@ -41537,7 +41537,7 @@
         <v>330000</v>
       </c>
       <c r="X130" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y130" s="54" t="n">
         <v>5</v>
@@ -41846,7 +41846,7 @@
         <v>330000</v>
       </c>
       <c r="X131" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y131" s="54" t="n">
         <v>5</v>
@@ -42155,7 +42155,7 @@
         <v>330000</v>
       </c>
       <c r="X132" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y132" s="54" t="n">
         <v>5</v>
@@ -42464,7 +42464,7 @@
         <v>330000</v>
       </c>
       <c r="X133" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y133" s="54" t="n">
         <v>5</v>
@@ -42773,7 +42773,7 @@
         <v>330000</v>
       </c>
       <c r="X134" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y134" s="54" t="n">
         <v>5</v>
@@ -43082,7 +43082,7 @@
         <v>330000</v>
       </c>
       <c r="X135" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y135" s="54" t="n">
         <v>5</v>
@@ -43391,7 +43391,7 @@
         <v>330000</v>
       </c>
       <c r="X136" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y136" s="54" t="n">
         <v>5</v>
@@ -43700,7 +43700,7 @@
         <v>330000</v>
       </c>
       <c r="X137" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y137" s="54" t="n">
         <v>5</v>
@@ -44009,7 +44009,7 @@
         <v>330000</v>
       </c>
       <c r="X138" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y138" s="54" t="n">
         <v>5</v>
@@ -44318,7 +44318,7 @@
         <v>330000</v>
       </c>
       <c r="X139" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y139" s="54" t="n">
         <v>5</v>
@@ -44627,7 +44627,7 @@
         <v>330000</v>
       </c>
       <c r="X140" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y140" s="54" t="n">
         <v>5</v>
@@ -44936,7 +44936,7 @@
         <v>330000</v>
       </c>
       <c r="X141" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y141" s="54" t="n">
         <v>5</v>
@@ -45245,7 +45245,7 @@
         <v>330000</v>
       </c>
       <c r="X142" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y142" s="54" t="n">
         <v>5</v>
@@ -45554,7 +45554,7 @@
         <v>330000</v>
       </c>
       <c r="X143" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y143" s="54" t="n">
         <v>5</v>
@@ -45863,7 +45863,7 @@
         <v>330000</v>
       </c>
       <c r="X144" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y144" s="54" t="n">
         <v>5</v>
@@ -46172,7 +46172,7 @@
         <v>330000</v>
       </c>
       <c r="X145" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y145" s="54" t="n">
         <v>5</v>
@@ -46481,7 +46481,7 @@
         <v>330000</v>
       </c>
       <c r="X146" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y146" s="54" t="n">
         <v>5</v>
@@ -46790,7 +46790,7 @@
         <v>330000</v>
       </c>
       <c r="X147" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y147" s="54" t="n">
         <v>5</v>
@@ -47099,7 +47099,7 @@
         <v>330000</v>
       </c>
       <c r="X148" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y148" s="54" t="n">
         <v>5</v>
@@ -47408,7 +47408,7 @@
         <v>330000</v>
       </c>
       <c r="X149" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y149" s="54" t="n">
         <v>5</v>
@@ -47717,7 +47717,7 @@
         <v>330000</v>
       </c>
       <c r="X150" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y150" s="54" t="n">
         <v>5</v>
@@ -48026,7 +48026,7 @@
         <v>330000</v>
       </c>
       <c r="X151" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y151" s="54" t="n">
         <v>5</v>
@@ -48335,7 +48335,7 @@
         <v>330000</v>
       </c>
       <c r="X152" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y152" s="54" t="n">
         <v>5</v>
@@ -48644,7 +48644,7 @@
         <v>330000</v>
       </c>
       <c r="X153" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y153" s="54" t="n">
         <v>5</v>
@@ -48953,7 +48953,7 @@
         <v>330000</v>
       </c>
       <c r="X154" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y154" s="54" t="n">
         <v>5</v>
@@ -49262,7 +49262,7 @@
         <v>330000</v>
       </c>
       <c r="X155" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y155" s="54" t="n">
         <v>5</v>
@@ -49571,7 +49571,7 @@
         <v>330000</v>
       </c>
       <c r="X156" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y156" s="54" t="n">
         <v>5</v>
@@ -49880,7 +49880,7 @@
         <v>330000</v>
       </c>
       <c r="X157" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y157" s="54" t="n">
         <v>5</v>
@@ -50189,7 +50189,7 @@
         <v>330000</v>
       </c>
       <c r="X158" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y158" s="54" t="n">
         <v>5</v>
@@ -50498,7 +50498,7 @@
         <v>330000</v>
       </c>
       <c r="X159" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y159" s="54" t="n">
         <v>5</v>
@@ -50807,7 +50807,7 @@
         <v>330000</v>
       </c>
       <c r="X160" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y160" s="54" t="n">
         <v>5</v>
@@ -51116,7 +51116,7 @@
         <v>330000</v>
       </c>
       <c r="X161" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y161" s="54" t="n">
         <v>5</v>
@@ -51425,7 +51425,7 @@
         <v>330000</v>
       </c>
       <c r="X162" s="54" t="n">
-        <v>26400</v>
+        <v>16500</v>
       </c>
       <c r="Y162" s="54" t="n">
         <v>5</v>
@@ -51734,7 +51734,7 @@
         <v>660000</v>
       </c>
       <c r="X163" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y163" s="54" t="n">
         <v>10</v>
@@ -52043,7 +52043,7 @@
         <v>660000</v>
       </c>
       <c r="X164" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y164" s="54" t="n">
         <v>10</v>
@@ -52352,7 +52352,7 @@
         <v>660000</v>
       </c>
       <c r="X165" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y165" s="54" t="n">
         <v>10</v>
@@ -52661,7 +52661,7 @@
         <v>660000</v>
       </c>
       <c r="X166" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y166" s="54" t="n">
         <v>10</v>
@@ -52970,7 +52970,7 @@
         <v>660000</v>
       </c>
       <c r="X167" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y167" s="54" t="n">
         <v>10</v>
@@ -53279,7 +53279,7 @@
         <v>660000</v>
       </c>
       <c r="X168" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y168" s="54" t="n">
         <v>10</v>
@@ -53588,7 +53588,7 @@
         <v>660000</v>
       </c>
       <c r="X169" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y169" s="54" t="n">
         <v>10</v>
@@ -53897,7 +53897,7 @@
         <v>660000</v>
       </c>
       <c r="X170" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y170" s="54" t="n">
         <v>10</v>
@@ -54206,7 +54206,7 @@
         <v>660000</v>
       </c>
       <c r="X171" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y171" s="54" t="n">
         <v>10</v>
@@ -54515,7 +54515,7 @@
         <v>660000</v>
       </c>
       <c r="X172" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y172" s="54" t="n">
         <v>10</v>
@@ -54824,7 +54824,7 @@
         <v>660000</v>
       </c>
       <c r="X173" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y173" s="54" t="n">
         <v>10</v>
@@ -55133,7 +55133,7 @@
         <v>660000</v>
       </c>
       <c r="X174" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y174" s="54" t="n">
         <v>10</v>
@@ -55442,7 +55442,7 @@
         <v>660000</v>
       </c>
       <c r="X175" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y175" s="54" t="n">
         <v>10</v>
@@ -55751,7 +55751,7 @@
         <v>660000</v>
       </c>
       <c r="X176" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y176" s="54" t="n">
         <v>10</v>
@@ -56060,7 +56060,7 @@
         <v>660000</v>
       </c>
       <c r="X177" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y177" s="54" t="n">
         <v>10</v>
@@ -56369,7 +56369,7 @@
         <v>660000</v>
       </c>
       <c r="X178" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y178" s="54" t="n">
         <v>10</v>
@@ -56678,7 +56678,7 @@
         <v>660000</v>
       </c>
       <c r="X179" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y179" s="54" t="n">
         <v>10</v>
@@ -56987,7 +56987,7 @@
         <v>660000</v>
       </c>
       <c r="X180" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y180" s="54" t="n">
         <v>10</v>
@@ -57296,7 +57296,7 @@
         <v>660000</v>
       </c>
       <c r="X181" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y181" s="54" t="n">
         <v>10</v>
@@ -57605,7 +57605,7 @@
         <v>660000</v>
       </c>
       <c r="X182" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y182" s="54" t="n">
         <v>10</v>
@@ -57914,7 +57914,7 @@
         <v>660000</v>
       </c>
       <c r="X183" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y183" s="54" t="n">
         <v>10</v>
@@ -58223,7 +58223,7 @@
         <v>660000</v>
       </c>
       <c r="X184" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y184" s="54" t="n">
         <v>10</v>
@@ -58532,7 +58532,7 @@
         <v>660000</v>
       </c>
       <c r="X185" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y185" s="54" t="n">
         <v>10</v>
@@ -58841,7 +58841,7 @@
         <v>660000</v>
       </c>
       <c r="X186" s="54" t="n">
-        <v>52800</v>
+        <v>33000</v>
       </c>
       <c r="Y186" s="54" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Recatégoriser 30 prescripteurs CORE (classe B d'origine) en NON CORE
- 30 derniers CORE de classe B (DrName) passés en NON CORE
- Recalcul: visite 1, TP=330000, BUS=16500 (5%), PPD=5
- Résultat: 69 CORE + 115 NON CORE = 184 lignes

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alpha_Kebe liste des prescripteur.xlsx
+++ b/Alpha_Kebe liste des prescripteur.xlsx
@@ -35322,11 +35322,11 @@
         </is>
       </c>
       <c r="M110" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N110" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O110" s="51" t="inlineStr">
@@ -35354,13 +35354,13 @@
       <c r="U110" s="65" t="n"/>
       <c r="V110" s="57" t="n"/>
       <c r="W110" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X110" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y110" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z110" s="43" t="n"/>
       <c r="AA110" s="43" t="n"/>
@@ -35631,11 +35631,11 @@
         </is>
       </c>
       <c r="M111" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N111" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O111" s="51" t="inlineStr">
@@ -35663,13 +35663,13 @@
       <c r="U111" s="65" t="n"/>
       <c r="V111" s="57" t="n"/>
       <c r="W111" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X111" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y111" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z111" s="43" t="n"/>
       <c r="AA111" s="43" t="n"/>
@@ -36249,11 +36249,11 @@
         </is>
       </c>
       <c r="M113" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N113" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O113" s="51" t="inlineStr">
@@ -36281,13 +36281,13 @@
       <c r="U113" s="65" t="n"/>
       <c r="V113" s="57" t="n"/>
       <c r="W113" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X113" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y113" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z113" s="43" t="n"/>
       <c r="AA113" s="43" t="n"/>
@@ -36558,11 +36558,11 @@
         </is>
       </c>
       <c r="M114" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N114" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O114" s="51" t="inlineStr">
@@ -36590,13 +36590,13 @@
       <c r="U114" s="65" t="n"/>
       <c r="V114" s="57" t="n"/>
       <c r="W114" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X114" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y114" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z114" s="43" t="n"/>
       <c r="AA114" s="43" t="n"/>
@@ -36867,11 +36867,11 @@
         </is>
       </c>
       <c r="M115" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N115" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O115" s="51" t="inlineStr">
@@ -36899,13 +36899,13 @@
       <c r="U115" s="65" t="n"/>
       <c r="V115" s="57" t="n"/>
       <c r="W115" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X115" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y115" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z115" s="43" t="n"/>
       <c r="AA115" s="43" t="n"/>
@@ -38103,11 +38103,11 @@
         </is>
       </c>
       <c r="M119" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N119" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O119" s="51" t="inlineStr">
@@ -38135,13 +38135,13 @@
       <c r="U119" s="65" t="n"/>
       <c r="V119" s="57" t="n"/>
       <c r="W119" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X119" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y119" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z119" s="43" t="n"/>
       <c r="AA119" s="43" t="n"/>
@@ -38412,11 +38412,11 @@
         </is>
       </c>
       <c r="M120" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N120" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O120" s="51" t="inlineStr">
@@ -38444,13 +38444,13 @@
       <c r="U120" s="65" t="n"/>
       <c r="V120" s="57" t="n"/>
       <c r="W120" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X120" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y120" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z120" s="43" t="n"/>
       <c r="AA120" s="43" t="n"/>
@@ -38721,11 +38721,11 @@
         </is>
       </c>
       <c r="M121" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N121" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O121" s="51" t="inlineStr">
@@ -38753,13 +38753,13 @@
       <c r="U121" s="65" t="n"/>
       <c r="V121" s="57" t="n"/>
       <c r="W121" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X121" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y121" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z121" s="43" t="n"/>
       <c r="AA121" s="43" t="n"/>
@@ -39030,11 +39030,11 @@
         </is>
       </c>
       <c r="M122" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N122" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O122" s="51" t="inlineStr">
@@ -39062,13 +39062,13 @@
       <c r="U122" s="65" t="n"/>
       <c r="V122" s="57" t="n"/>
       <c r="W122" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X122" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y122" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z122" s="43" t="n"/>
       <c r="AA122" s="43" t="n"/>
@@ -39648,11 +39648,11 @@
         </is>
       </c>
       <c r="M124" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N124" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O124" s="51" t="inlineStr">
@@ -39680,13 +39680,13 @@
       <c r="U124" s="65" t="n"/>
       <c r="V124" s="57" t="n"/>
       <c r="W124" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X124" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y124" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z124" s="43" t="n"/>
       <c r="AA124" s="43" t="n"/>
@@ -40266,11 +40266,11 @@
         </is>
       </c>
       <c r="M126" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N126" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O126" s="51" t="inlineStr">
@@ -40298,13 +40298,13 @@
       <c r="U126" s="65" t="n"/>
       <c r="V126" s="57" t="n"/>
       <c r="W126" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X126" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y126" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z126" s="43" t="n"/>
       <c r="AA126" s="43" t="n"/>
@@ -52008,11 +52008,11 @@
         </is>
       </c>
       <c r="M164" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N164" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O164" s="51" t="inlineStr">
@@ -52040,13 +52040,13 @@
       <c r="U164" s="65" t="n"/>
       <c r="V164" s="57" t="n"/>
       <c r="W164" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X164" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y164" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z164" s="43" t="n"/>
       <c r="AA164" s="43" t="n"/>
@@ -52626,11 +52626,11 @@
         </is>
       </c>
       <c r="M166" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N166" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O166" s="51" t="inlineStr">
@@ -52658,13 +52658,13 @@
       <c r="U166" s="65" t="n"/>
       <c r="V166" s="57" t="n"/>
       <c r="W166" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X166" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y166" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z166" s="43" t="n"/>
       <c r="AA166" s="43" t="n"/>
@@ -52935,11 +52935,11 @@
         </is>
       </c>
       <c r="M167" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N167" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O167" s="51" t="inlineStr">
@@ -52967,13 +52967,13 @@
       <c r="U167" s="65" t="n"/>
       <c r="V167" s="57" t="n"/>
       <c r="W167" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X167" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y167" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z167" s="43" t="n"/>
       <c r="AA167" s="43" t="n"/>
@@ -53244,11 +53244,11 @@
         </is>
       </c>
       <c r="M168" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N168" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O168" s="51" t="inlineStr">
@@ -53276,13 +53276,13 @@
       <c r="U168" s="65" t="n"/>
       <c r="V168" s="57" t="n"/>
       <c r="W168" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X168" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y168" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z168" s="43" t="n"/>
       <c r="AA168" s="43" t="n"/>
@@ -53553,11 +53553,11 @@
         </is>
       </c>
       <c r="M169" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N169" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O169" s="51" t="inlineStr">
@@ -53585,13 +53585,13 @@
       <c r="U169" s="65" t="n"/>
       <c r="V169" s="57" t="n"/>
       <c r="W169" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X169" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y169" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z169" s="43" t="n"/>
       <c r="AA169" s="43" t="n"/>
@@ -53862,11 +53862,11 @@
         </is>
       </c>
       <c r="M170" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N170" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O170" s="51" t="inlineStr">
@@ -53894,13 +53894,13 @@
       <c r="U170" s="65" t="n"/>
       <c r="V170" s="57" t="n"/>
       <c r="W170" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X170" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y170" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z170" s="43" t="n"/>
       <c r="AA170" s="43" t="n"/>
@@ -54480,11 +54480,11 @@
         </is>
       </c>
       <c r="M172" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N172" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O172" s="51" t="inlineStr">
@@ -54512,13 +54512,13 @@
       <c r="U172" s="65" t="n"/>
       <c r="V172" s="57" t="n"/>
       <c r="W172" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X172" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y172" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z172" s="43" t="n"/>
       <c r="AA172" s="43" t="n"/>
@@ -54789,11 +54789,11 @@
         </is>
       </c>
       <c r="M173" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N173" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O173" s="51" t="inlineStr">
@@ -54821,13 +54821,13 @@
       <c r="U173" s="65" t="n"/>
       <c r="V173" s="57" t="n"/>
       <c r="W173" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X173" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y173" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z173" s="43" t="n"/>
       <c r="AA173" s="43" t="n"/>
@@ -55098,11 +55098,11 @@
         </is>
       </c>
       <c r="M174" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N174" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O174" s="51" t="inlineStr">
@@ -55130,13 +55130,13 @@
       <c r="U174" s="65" t="n"/>
       <c r="V174" s="57" t="n"/>
       <c r="W174" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X174" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y174" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z174" s="43" t="n"/>
       <c r="AA174" s="43" t="n"/>
@@ -55407,11 +55407,11 @@
         </is>
       </c>
       <c r="M175" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N175" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O175" s="51" t="inlineStr">
@@ -55439,13 +55439,13 @@
       <c r="U175" s="65" t="n"/>
       <c r="V175" s="57" t="n"/>
       <c r="W175" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X175" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y175" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z175" s="43" t="n"/>
       <c r="AA175" s="43" t="n"/>
@@ -56025,11 +56025,11 @@
         </is>
       </c>
       <c r="M177" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N177" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O177" s="51" t="inlineStr">
@@ -56057,13 +56057,13 @@
       <c r="U177" s="65" t="n"/>
       <c r="V177" s="57" t="n"/>
       <c r="W177" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X177" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y177" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z177" s="43" t="n"/>
       <c r="AA177" s="43" t="n"/>
@@ -56334,11 +56334,11 @@
         </is>
       </c>
       <c r="M178" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N178" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O178" s="51" t="inlineStr">
@@ -56366,13 +56366,13 @@
       <c r="U178" s="65" t="n"/>
       <c r="V178" s="57" t="n"/>
       <c r="W178" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X178" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y178" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z178" s="43" t="n"/>
       <c r="AA178" s="43" t="n"/>
@@ -56643,11 +56643,11 @@
         </is>
       </c>
       <c r="M179" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N179" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O179" s="51" t="inlineStr">
@@ -56675,13 +56675,13 @@
       <c r="U179" s="65" t="n"/>
       <c r="V179" s="57" t="n"/>
       <c r="W179" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X179" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y179" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z179" s="43" t="n"/>
       <c r="AA179" s="43" t="n"/>
@@ -56952,11 +56952,11 @@
         </is>
       </c>
       <c r="M180" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N180" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O180" s="51" t="inlineStr">
@@ -56984,13 +56984,13 @@
       <c r="U180" s="65" t="n"/>
       <c r="V180" s="57" t="n"/>
       <c r="W180" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X180" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y180" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z180" s="43" t="n"/>
       <c r="AA180" s="43" t="n"/>
@@ -57261,11 +57261,11 @@
         </is>
       </c>
       <c r="M181" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N181" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O181" s="51" t="inlineStr">
@@ -57293,13 +57293,13 @@
       <c r="U181" s="65" t="n"/>
       <c r="V181" s="57" t="n"/>
       <c r="W181" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X181" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y181" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z181" s="43" t="n"/>
       <c r="AA181" s="43" t="n"/>
@@ -57570,11 +57570,11 @@
         </is>
       </c>
       <c r="M182" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N182" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O182" s="51" t="inlineStr">
@@ -57602,13 +57602,13 @@
       <c r="U182" s="65" t="n"/>
       <c r="V182" s="57" t="n"/>
       <c r="W182" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X182" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y182" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z182" s="43" t="n"/>
       <c r="AA182" s="43" t="n"/>
@@ -57879,11 +57879,11 @@
         </is>
       </c>
       <c r="M183" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N183" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O183" s="51" t="inlineStr">
@@ -57911,13 +57911,13 @@
       <c r="U183" s="65" t="n"/>
       <c r="V183" s="57" t="n"/>
       <c r="W183" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X183" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y183" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z183" s="43" t="n"/>
       <c r="AA183" s="43" t="n"/>
@@ -58497,11 +58497,11 @@
         </is>
       </c>
       <c r="M185" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N185" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O185" s="51" t="inlineStr">
@@ -58529,13 +58529,13 @@
       <c r="U185" s="65" t="n"/>
       <c r="V185" s="57" t="n"/>
       <c r="W185" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X185" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y185" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z185" s="43" t="n"/>
       <c r="AA185" s="43" t="n"/>
@@ -58806,11 +58806,11 @@
         </is>
       </c>
       <c r="M186" s="51" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N186" s="51" t="inlineStr">
         <is>
-          <t>CORE</t>
+          <t>NON CORE</t>
         </is>
       </c>
       <c r="O186" s="51" t="inlineStr">
@@ -58838,13 +58838,13 @@
       <c r="U186" s="65" t="n"/>
       <c r="V186" s="57" t="n"/>
       <c r="W186" s="54" t="n">
-        <v>660000</v>
+        <v>330000</v>
       </c>
       <c r="X186" s="54" t="n">
-        <v>33000</v>
+        <v>16500</v>
       </c>
       <c r="Y186" s="54" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="Z186" s="43" t="n"/>
       <c r="AA186" s="43" t="n"/>

</xml_diff>

<commit_message>
NO OF VISIT des CORE entre 2 et 3 selon la classe d'origine
- Classe A+ / A: 3 visites (55 prescripteurs)
- Classe B: 2 visites (14 prescripteurs)
- NON CORE inchangés à 1 visite

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alpha_Kebe liste des prescripteur.xlsx
+++ b/Alpha_Kebe liste des prescripteur.xlsx
@@ -27292,7 +27292,7 @@
         </is>
       </c>
       <c r="M84" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N84" s="51" t="inlineStr">
         <is>
@@ -27600,7 +27600,7 @@
         </is>
       </c>
       <c r="M85" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N85" s="51" t="inlineStr">
         <is>
@@ -27908,7 +27908,7 @@
         </is>
       </c>
       <c r="M86" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N86" s="51" t="inlineStr">
         <is>
@@ -28833,7 +28833,7 @@
         </is>
       </c>
       <c r="M89" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N89" s="51" t="inlineStr">
         <is>
@@ -29142,7 +29142,7 @@
         </is>
       </c>
       <c r="M90" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N90" s="51" t="inlineStr">
         <is>
@@ -29760,7 +29760,7 @@
         </is>
       </c>
       <c r="M92" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N92" s="51" t="inlineStr">
         <is>
@@ -30378,7 +30378,7 @@
         </is>
       </c>
       <c r="M94" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N94" s="51" t="inlineStr">
         <is>
@@ -30687,7 +30687,7 @@
         </is>
       </c>
       <c r="M95" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N95" s="51" t="inlineStr">
         <is>
@@ -31923,7 +31923,7 @@
         </is>
       </c>
       <c r="M99" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N99" s="51" t="inlineStr">
         <is>
@@ -32541,7 +32541,7 @@
         </is>
       </c>
       <c r="M101" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N101" s="51" t="inlineStr">
         <is>
@@ -33159,7 +33159,7 @@
         </is>
       </c>
       <c r="M103" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N103" s="51" t="inlineStr">
         <is>
@@ -33468,7 +33468,7 @@
         </is>
       </c>
       <c r="M104" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N104" s="51" t="inlineStr">
         <is>
@@ -34395,7 +34395,7 @@
         </is>
       </c>
       <c r="M107" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N107" s="51" t="inlineStr">
         <is>
@@ -35013,7 +35013,7 @@
         </is>
       </c>
       <c r="M109" s="51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N109" s="51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
BUS TO DIV: passer de 5% à 3% du TOTAL_POTENTIAL
- CORE: 660000 x 3% = 19800 (69 lignes)
- NON CORE: 330000 x 3% = 9900 (115 lignes)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Alpha_Kebe liste des prescripteur.xlsx
+++ b/Alpha_Kebe liste des prescripteur.xlsx
@@ -2579,7 +2579,7 @@
         <v>330000</v>
       </c>
       <c r="X3" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y3" s="54" t="n">
         <v>5</v>
@@ -2668,7 +2668,7 @@
         <v>330000</v>
       </c>
       <c r="X4" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y4" s="54" t="n">
         <v>5</v>
@@ -2977,7 +2977,7 @@
         <v>330000</v>
       </c>
       <c r="X5" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y5" s="54" t="n">
         <v>5</v>
@@ -3286,7 +3286,7 @@
         <v>330000</v>
       </c>
       <c r="X6" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y6" s="54" t="n">
         <v>5</v>
@@ -3595,7 +3595,7 @@
         <v>660000</v>
       </c>
       <c r="X7" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y7" s="54" t="n">
         <v>10</v>
@@ -3904,7 +3904,7 @@
         <v>660000</v>
       </c>
       <c r="X8" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y8" s="54" t="n">
         <v>10</v>
@@ -4213,7 +4213,7 @@
         <v>330000</v>
       </c>
       <c r="X9" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y9" s="54" t="n">
         <v>5</v>
@@ -4522,7 +4522,7 @@
         <v>330000</v>
       </c>
       <c r="X10" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y10" s="54" t="n">
         <v>5</v>
@@ -4831,7 +4831,7 @@
         <v>330000</v>
       </c>
       <c r="X11" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y11" s="54" t="n">
         <v>5</v>
@@ -5140,7 +5140,7 @@
         <v>660000</v>
       </c>
       <c r="X12" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y12" s="54" t="n">
         <v>10</v>
@@ -5449,7 +5449,7 @@
         <v>660000</v>
       </c>
       <c r="X13" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y13" s="54" t="n">
         <v>10</v>
@@ -5758,7 +5758,7 @@
         <v>660000</v>
       </c>
       <c r="X14" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y14" s="54" t="n">
         <v>10</v>
@@ -6067,7 +6067,7 @@
         <v>660000</v>
       </c>
       <c r="X15" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y15" s="54" t="n">
         <v>10</v>
@@ -6376,7 +6376,7 @@
         <v>660000</v>
       </c>
       <c r="X16" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y16" s="54" t="n">
         <v>10</v>
@@ -6685,7 +6685,7 @@
         <v>330000</v>
       </c>
       <c r="X17" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y17" s="54" t="n">
         <v>5</v>
@@ -6993,7 +6993,7 @@
         <v>330000</v>
       </c>
       <c r="X18" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y18" s="54" t="n">
         <v>5</v>
@@ -7302,7 +7302,7 @@
         <v>660000</v>
       </c>
       <c r="X19" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y19" s="54" t="n">
         <v>10</v>
@@ -7611,7 +7611,7 @@
         <v>660000</v>
       </c>
       <c r="X20" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y20" s="54" t="n">
         <v>10</v>
@@ -7920,7 +7920,7 @@
         <v>660000</v>
       </c>
       <c r="X21" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y21" s="54" t="n">
         <v>10</v>
@@ -8229,7 +8229,7 @@
         <v>660000</v>
       </c>
       <c r="X22" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y22" s="54" t="n">
         <v>10</v>
@@ -8538,7 +8538,7 @@
         <v>660000</v>
       </c>
       <c r="X23" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y23" s="54" t="n">
         <v>10</v>
@@ -8846,7 +8846,7 @@
         <v>660000</v>
       </c>
       <c r="X24" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y24" s="54" t="n">
         <v>10</v>
@@ -9154,7 +9154,7 @@
         <v>660000</v>
       </c>
       <c r="X25" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y25" s="54" t="n">
         <v>10</v>
@@ -9462,7 +9462,7 @@
         <v>330000</v>
       </c>
       <c r="X26" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y26" s="54" t="n">
         <v>5</v>
@@ -9770,7 +9770,7 @@
         <v>660000</v>
       </c>
       <c r="X27" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y27" s="54" t="n">
         <v>10</v>
@@ -10078,7 +10078,7 @@
         <v>660000</v>
       </c>
       <c r="X28" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y28" s="54" t="n">
         <v>10</v>
@@ -10386,7 +10386,7 @@
         <v>330000</v>
       </c>
       <c r="X29" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y29" s="54" t="n">
         <v>5</v>
@@ -10694,7 +10694,7 @@
         <v>330000</v>
       </c>
       <c r="X30" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y30" s="54" t="n">
         <v>5</v>
@@ -11002,7 +11002,7 @@
         <v>330000</v>
       </c>
       <c r="X31" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y31" s="54" t="n">
         <v>5</v>
@@ -11310,7 +11310,7 @@
         <v>330000</v>
       </c>
       <c r="X32" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y32" s="54" t="n">
         <v>5</v>
@@ -11618,7 +11618,7 @@
         <v>660000</v>
       </c>
       <c r="X33" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y33" s="54" t="n">
         <v>10</v>
@@ -11926,7 +11926,7 @@
         <v>660000</v>
       </c>
       <c r="X34" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y34" s="54" t="n">
         <v>10</v>
@@ -12234,7 +12234,7 @@
         <v>660000</v>
       </c>
       <c r="X35" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y35" s="54" t="n">
         <v>10</v>
@@ -12542,7 +12542,7 @@
         <v>660000</v>
       </c>
       <c r="X36" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y36" s="54" t="n">
         <v>10</v>
@@ -12850,7 +12850,7 @@
         <v>660000</v>
       </c>
       <c r="X37" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y37" s="54" t="n">
         <v>10</v>
@@ -13158,7 +13158,7 @@
         <v>330000</v>
       </c>
       <c r="X38" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y38" s="54" t="n">
         <v>5</v>
@@ -13466,7 +13466,7 @@
         <v>660000</v>
       </c>
       <c r="X39" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y39" s="54" t="n">
         <v>10</v>
@@ -13774,7 +13774,7 @@
         <v>660000</v>
       </c>
       <c r="X40" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y40" s="54" t="n">
         <v>10</v>
@@ -14082,7 +14082,7 @@
         <v>660000</v>
       </c>
       <c r="X41" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y41" s="54" t="n">
         <v>10</v>
@@ -14390,7 +14390,7 @@
         <v>660000</v>
       </c>
       <c r="X42" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y42" s="54" t="n">
         <v>10</v>
@@ -14698,7 +14698,7 @@
         <v>660000</v>
       </c>
       <c r="X43" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y43" s="54" t="n">
         <v>10</v>
@@ -15006,7 +15006,7 @@
         <v>330000</v>
       </c>
       <c r="X44" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y44" s="54" t="n">
         <v>5</v>
@@ -15314,7 +15314,7 @@
         <v>660000</v>
       </c>
       <c r="X45" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y45" s="54" t="n">
         <v>10</v>
@@ -15622,7 +15622,7 @@
         <v>660000</v>
       </c>
       <c r="X46" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y46" s="54" t="n">
         <v>10</v>
@@ -15930,7 +15930,7 @@
         <v>330000</v>
       </c>
       <c r="X47" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y47" s="54" t="n">
         <v>5</v>
@@ -16238,7 +16238,7 @@
         <v>330000</v>
       </c>
       <c r="X48" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y48" s="54" t="n">
         <v>5</v>
@@ -16546,7 +16546,7 @@
         <v>330000</v>
       </c>
       <c r="X49" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y49" s="54" t="n">
         <v>5</v>
@@ -16854,7 +16854,7 @@
         <v>330000</v>
       </c>
       <c r="X50" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y50" s="54" t="n">
         <v>5</v>
@@ -17162,7 +17162,7 @@
         <v>330000</v>
       </c>
       <c r="X51" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y51" s="54" t="n">
         <v>5</v>
@@ -17470,7 +17470,7 @@
         <v>330000</v>
       </c>
       <c r="X52" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y52" s="54" t="n">
         <v>5</v>
@@ -17778,7 +17778,7 @@
         <v>330000</v>
       </c>
       <c r="X53" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y53" s="54" t="n">
         <v>5</v>
@@ -18086,7 +18086,7 @@
         <v>330000</v>
       </c>
       <c r="X54" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y54" s="54" t="n">
         <v>5</v>
@@ -18394,7 +18394,7 @@
         <v>330000</v>
       </c>
       <c r="X55" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y55" s="54" t="n">
         <v>5</v>
@@ -18702,7 +18702,7 @@
         <v>330000</v>
       </c>
       <c r="X56" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y56" s="54" t="n">
         <v>5</v>
@@ -19010,7 +19010,7 @@
         <v>330000</v>
       </c>
       <c r="X57" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y57" s="54" t="n">
         <v>5</v>
@@ -19318,7 +19318,7 @@
         <v>330000</v>
       </c>
       <c r="X58" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y58" s="54" t="n">
         <v>5</v>
@@ -19626,7 +19626,7 @@
         <v>330000</v>
       </c>
       <c r="X59" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y59" s="54" t="n">
         <v>5</v>
@@ -19934,7 +19934,7 @@
         <v>660000</v>
       </c>
       <c r="X60" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y60" s="54" t="n">
         <v>10</v>
@@ -20242,7 +20242,7 @@
         <v>660000</v>
       </c>
       <c r="X61" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y61" s="54" t="n">
         <v>10</v>
@@ -20550,7 +20550,7 @@
         <v>660000</v>
       </c>
       <c r="X62" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y62" s="54" t="n">
         <v>10</v>
@@ -20858,7 +20858,7 @@
         <v>330000</v>
       </c>
       <c r="X63" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y63" s="54" t="n">
         <v>5</v>
@@ -21166,7 +21166,7 @@
         <v>330000</v>
       </c>
       <c r="X64" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y64" s="54" t="n">
         <v>5</v>
@@ -21474,7 +21474,7 @@
         <v>330000</v>
       </c>
       <c r="X65" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y65" s="54" t="n">
         <v>5</v>
@@ -21782,7 +21782,7 @@
         <v>660000</v>
       </c>
       <c r="X66" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y66" s="54" t="n">
         <v>10</v>
@@ -22090,7 +22090,7 @@
         <v>330000</v>
       </c>
       <c r="X67" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y67" s="54" t="n">
         <v>5</v>
@@ -22398,7 +22398,7 @@
         <v>330000</v>
       </c>
       <c r="X68" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y68" s="54" t="n">
         <v>5</v>
@@ -22706,7 +22706,7 @@
         <v>330000</v>
       </c>
       <c r="X69" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y69" s="54" t="n">
         <v>5</v>
@@ -23014,7 +23014,7 @@
         <v>330000</v>
       </c>
       <c r="X70" s="43" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y70" s="54" t="n">
         <v>5</v>
@@ -23322,7 +23322,7 @@
         <v>660000</v>
       </c>
       <c r="X71" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y71" s="54" t="n">
         <v>10</v>
@@ -23630,7 +23630,7 @@
         <v>660000</v>
       </c>
       <c r="X72" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y72" s="54" t="n">
         <v>10</v>
@@ -23938,7 +23938,7 @@
         <v>660000</v>
       </c>
       <c r="X73" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y73" s="54" t="n">
         <v>10</v>
@@ -24247,7 +24247,7 @@
         <v>660000</v>
       </c>
       <c r="X74" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y74" s="54" t="n">
         <v>10</v>
@@ -24555,7 +24555,7 @@
         <v>660000</v>
       </c>
       <c r="X75" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y75" s="54" t="n">
         <v>10</v>
@@ -24863,7 +24863,7 @@
         <v>660000</v>
       </c>
       <c r="X76" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y76" s="54" t="n">
         <v>10</v>
@@ -25171,7 +25171,7 @@
         <v>660000</v>
       </c>
       <c r="X77" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y77" s="54" t="n">
         <v>10</v>
@@ -25479,7 +25479,7 @@
         <v>660000</v>
       </c>
       <c r="X78" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y78" s="54" t="n">
         <v>10</v>
@@ -25787,7 +25787,7 @@
         <v>660000</v>
       </c>
       <c r="X79" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y79" s="54" t="n">
         <v>10</v>
@@ -26095,7 +26095,7 @@
         <v>660000</v>
       </c>
       <c r="X80" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y80" s="54" t="n">
         <v>10</v>
@@ -26403,7 +26403,7 @@
         <v>660000</v>
       </c>
       <c r="X81" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y81" s="54" t="n">
         <v>10</v>
@@ -26711,7 +26711,7 @@
         <v>660000</v>
       </c>
       <c r="X82" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y82" s="54" t="n">
         <v>10</v>
@@ -27019,7 +27019,7 @@
         <v>660000</v>
       </c>
       <c r="X83" s="43" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y83" s="54" t="n">
         <v>10</v>
@@ -27327,7 +27327,7 @@
         <v>660000</v>
       </c>
       <c r="X84" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y84" s="54" t="n">
         <v>10</v>
@@ -27635,7 +27635,7 @@
         <v>660000</v>
       </c>
       <c r="X85" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y85" s="54" t="n">
         <v>10</v>
@@ -27943,7 +27943,7 @@
         <v>660000</v>
       </c>
       <c r="X86" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y86" s="54" t="n">
         <v>10</v>
@@ -28251,7 +28251,7 @@
         <v>330000</v>
       </c>
       <c r="X87" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y87" s="54" t="n">
         <v>5</v>
@@ -28559,7 +28559,7 @@
         <v>330000</v>
       </c>
       <c r="X88" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y88" s="54" t="n">
         <v>5</v>
@@ -28868,7 +28868,7 @@
         <v>660000</v>
       </c>
       <c r="X89" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y89" s="54" t="n">
         <v>10</v>
@@ -29177,7 +29177,7 @@
         <v>660000</v>
       </c>
       <c r="X90" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y90" s="54" t="n">
         <v>10</v>
@@ -29486,7 +29486,7 @@
         <v>330000</v>
       </c>
       <c r="X91" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y91" s="54" t="n">
         <v>5</v>
@@ -29795,7 +29795,7 @@
         <v>660000</v>
       </c>
       <c r="X92" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y92" s="54" t="n">
         <v>10</v>
@@ -30104,7 +30104,7 @@
         <v>330000</v>
       </c>
       <c r="X93" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y93" s="54" t="n">
         <v>5</v>
@@ -30413,7 +30413,7 @@
         <v>660000</v>
       </c>
       <c r="X94" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y94" s="54" t="n">
         <v>10</v>
@@ -30722,7 +30722,7 @@
         <v>660000</v>
       </c>
       <c r="X95" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y95" s="54" t="n">
         <v>10</v>
@@ -31031,7 +31031,7 @@
         <v>330000</v>
       </c>
       <c r="X96" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y96" s="54" t="n">
         <v>5</v>
@@ -31340,7 +31340,7 @@
         <v>330000</v>
       </c>
       <c r="X97" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y97" s="54" t="n">
         <v>5</v>
@@ -31649,7 +31649,7 @@
         <v>330000</v>
       </c>
       <c r="X98" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y98" s="54" t="n">
         <v>5</v>
@@ -31958,7 +31958,7 @@
         <v>660000</v>
       </c>
       <c r="X99" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y99" s="54" t="n">
         <v>10</v>
@@ -32267,7 +32267,7 @@
         <v>330000</v>
       </c>
       <c r="X100" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y100" s="54" t="n">
         <v>5</v>
@@ -32576,7 +32576,7 @@
         <v>660000</v>
       </c>
       <c r="X101" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y101" s="54" t="n">
         <v>10</v>
@@ -32885,7 +32885,7 @@
         <v>330000</v>
       </c>
       <c r="X102" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y102" s="54" t="n">
         <v>5</v>
@@ -33194,7 +33194,7 @@
         <v>660000</v>
       </c>
       <c r="X103" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y103" s="54" t="n">
         <v>10</v>
@@ -33503,7 +33503,7 @@
         <v>660000</v>
       </c>
       <c r="X104" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y104" s="54" t="n">
         <v>10</v>
@@ -33812,7 +33812,7 @@
         <v>330000</v>
       </c>
       <c r="X105" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y105" s="54" t="n">
         <v>5</v>
@@ -34121,7 +34121,7 @@
         <v>330000</v>
       </c>
       <c r="X106" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y106" s="54" t="n">
         <v>5</v>
@@ -34430,7 +34430,7 @@
         <v>660000</v>
       </c>
       <c r="X107" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y107" s="54" t="n">
         <v>10</v>
@@ -34739,7 +34739,7 @@
         <v>330000</v>
       </c>
       <c r="X108" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y108" s="54" t="n">
         <v>5</v>
@@ -35048,7 +35048,7 @@
         <v>660000</v>
       </c>
       <c r="X109" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y109" s="54" t="n">
         <v>10</v>
@@ -35357,7 +35357,7 @@
         <v>330000</v>
       </c>
       <c r="X110" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y110" s="54" t="n">
         <v>5</v>
@@ -35666,7 +35666,7 @@
         <v>330000</v>
       </c>
       <c r="X111" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y111" s="54" t="n">
         <v>5</v>
@@ -35975,7 +35975,7 @@
         <v>660000</v>
       </c>
       <c r="X112" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y112" s="54" t="n">
         <v>10</v>
@@ -36284,7 +36284,7 @@
         <v>330000</v>
       </c>
       <c r="X113" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y113" s="54" t="n">
         <v>5</v>
@@ -36593,7 +36593,7 @@
         <v>330000</v>
       </c>
       <c r="X114" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y114" s="54" t="n">
         <v>5</v>
@@ -36902,7 +36902,7 @@
         <v>330000</v>
       </c>
       <c r="X115" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y115" s="54" t="n">
         <v>5</v>
@@ -37211,7 +37211,7 @@
         <v>330000</v>
       </c>
       <c r="X116" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y116" s="54" t="n">
         <v>5</v>
@@ -37520,7 +37520,7 @@
         <v>660000</v>
       </c>
       <c r="X117" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y117" s="54" t="n">
         <v>10</v>
@@ -37829,7 +37829,7 @@
         <v>660000</v>
       </c>
       <c r="X118" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y118" s="54" t="n">
         <v>10</v>
@@ -38138,7 +38138,7 @@
         <v>330000</v>
       </c>
       <c r="X119" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y119" s="54" t="n">
         <v>5</v>
@@ -38447,7 +38447,7 @@
         <v>330000</v>
       </c>
       <c r="X120" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y120" s="54" t="n">
         <v>5</v>
@@ -38756,7 +38756,7 @@
         <v>330000</v>
       </c>
       <c r="X121" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y121" s="54" t="n">
         <v>5</v>
@@ -39065,7 +39065,7 @@
         <v>330000</v>
       </c>
       <c r="X122" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y122" s="54" t="n">
         <v>5</v>
@@ -39374,7 +39374,7 @@
         <v>330000</v>
       </c>
       <c r="X123" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y123" s="54" t="n">
         <v>5</v>
@@ -39683,7 +39683,7 @@
         <v>330000</v>
       </c>
       <c r="X124" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y124" s="54" t="n">
         <v>5</v>
@@ -39992,7 +39992,7 @@
         <v>660000</v>
       </c>
       <c r="X125" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y125" s="54" t="n">
         <v>10</v>
@@ -40301,7 +40301,7 @@
         <v>330000</v>
       </c>
       <c r="X126" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y126" s="54" t="n">
         <v>5</v>
@@ -40610,7 +40610,7 @@
         <v>330000</v>
       </c>
       <c r="X127" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y127" s="54" t="n">
         <v>5</v>
@@ -40919,7 +40919,7 @@
         <v>660000</v>
       </c>
       <c r="X128" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y128" s="54" t="n">
         <v>10</v>
@@ -41228,7 +41228,7 @@
         <v>330000</v>
       </c>
       <c r="X129" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y129" s="54" t="n">
         <v>5</v>
@@ -41537,7 +41537,7 @@
         <v>330000</v>
       </c>
       <c r="X130" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y130" s="54" t="n">
         <v>5</v>
@@ -41846,7 +41846,7 @@
         <v>330000</v>
       </c>
       <c r="X131" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y131" s="54" t="n">
         <v>5</v>
@@ -42155,7 +42155,7 @@
         <v>330000</v>
       </c>
       <c r="X132" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y132" s="54" t="n">
         <v>5</v>
@@ -42464,7 +42464,7 @@
         <v>330000</v>
       </c>
       <c r="X133" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y133" s="54" t="n">
         <v>5</v>
@@ -42773,7 +42773,7 @@
         <v>330000</v>
       </c>
       <c r="X134" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y134" s="54" t="n">
         <v>5</v>
@@ -43082,7 +43082,7 @@
         <v>330000</v>
       </c>
       <c r="X135" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y135" s="54" t="n">
         <v>5</v>
@@ -43391,7 +43391,7 @@
         <v>330000</v>
       </c>
       <c r="X136" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y136" s="54" t="n">
         <v>5</v>
@@ -43700,7 +43700,7 @@
         <v>330000</v>
       </c>
       <c r="X137" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y137" s="54" t="n">
         <v>5</v>
@@ -44009,7 +44009,7 @@
         <v>330000</v>
       </c>
       <c r="X138" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y138" s="54" t="n">
         <v>5</v>
@@ -44318,7 +44318,7 @@
         <v>330000</v>
       </c>
       <c r="X139" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y139" s="54" t="n">
         <v>5</v>
@@ -44627,7 +44627,7 @@
         <v>330000</v>
       </c>
       <c r="X140" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y140" s="54" t="n">
         <v>5</v>
@@ -44936,7 +44936,7 @@
         <v>330000</v>
       </c>
       <c r="X141" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y141" s="54" t="n">
         <v>5</v>
@@ -45245,7 +45245,7 @@
         <v>330000</v>
       </c>
       <c r="X142" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y142" s="54" t="n">
         <v>5</v>
@@ -45554,7 +45554,7 @@
         <v>330000</v>
       </c>
       <c r="X143" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y143" s="54" t="n">
         <v>5</v>
@@ -45863,7 +45863,7 @@
         <v>330000</v>
       </c>
       <c r="X144" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y144" s="54" t="n">
         <v>5</v>
@@ -46172,7 +46172,7 @@
         <v>330000</v>
       </c>
       <c r="X145" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y145" s="54" t="n">
         <v>5</v>
@@ -46481,7 +46481,7 @@
         <v>330000</v>
       </c>
       <c r="X146" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y146" s="54" t="n">
         <v>5</v>
@@ -46790,7 +46790,7 @@
         <v>330000</v>
       </c>
       <c r="X147" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y147" s="54" t="n">
         <v>5</v>
@@ -47099,7 +47099,7 @@
         <v>330000</v>
       </c>
       <c r="X148" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y148" s="54" t="n">
         <v>5</v>
@@ -47408,7 +47408,7 @@
         <v>330000</v>
       </c>
       <c r="X149" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y149" s="54" t="n">
         <v>5</v>
@@ -47717,7 +47717,7 @@
         <v>330000</v>
       </c>
       <c r="X150" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y150" s="54" t="n">
         <v>5</v>
@@ -48026,7 +48026,7 @@
         <v>330000</v>
       </c>
       <c r="X151" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y151" s="54" t="n">
         <v>5</v>
@@ -48335,7 +48335,7 @@
         <v>330000</v>
       </c>
       <c r="X152" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y152" s="54" t="n">
         <v>5</v>
@@ -48644,7 +48644,7 @@
         <v>330000</v>
       </c>
       <c r="X153" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y153" s="54" t="n">
         <v>5</v>
@@ -48953,7 +48953,7 @@
         <v>330000</v>
       </c>
       <c r="X154" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y154" s="54" t="n">
         <v>5</v>
@@ -49262,7 +49262,7 @@
         <v>330000</v>
       </c>
       <c r="X155" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y155" s="54" t="n">
         <v>5</v>
@@ -49571,7 +49571,7 @@
         <v>330000</v>
       </c>
       <c r="X156" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y156" s="54" t="n">
         <v>5</v>
@@ -49880,7 +49880,7 @@
         <v>330000</v>
       </c>
       <c r="X157" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y157" s="54" t="n">
         <v>5</v>
@@ -50189,7 +50189,7 @@
         <v>330000</v>
       </c>
       <c r="X158" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y158" s="54" t="n">
         <v>5</v>
@@ -50498,7 +50498,7 @@
         <v>330000</v>
       </c>
       <c r="X159" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y159" s="54" t="n">
         <v>5</v>
@@ -50807,7 +50807,7 @@
         <v>330000</v>
       </c>
       <c r="X160" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y160" s="54" t="n">
         <v>5</v>
@@ -51116,7 +51116,7 @@
         <v>330000</v>
       </c>
       <c r="X161" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y161" s="54" t="n">
         <v>5</v>
@@ -51425,7 +51425,7 @@
         <v>330000</v>
       </c>
       <c r="X162" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y162" s="54" t="n">
         <v>5</v>
@@ -51734,7 +51734,7 @@
         <v>660000</v>
       </c>
       <c r="X163" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y163" s="54" t="n">
         <v>10</v>
@@ -52043,7 +52043,7 @@
         <v>330000</v>
       </c>
       <c r="X164" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y164" s="54" t="n">
         <v>5</v>
@@ -52352,7 +52352,7 @@
         <v>660000</v>
       </c>
       <c r="X165" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y165" s="54" t="n">
         <v>10</v>
@@ -52661,7 +52661,7 @@
         <v>330000</v>
       </c>
       <c r="X166" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y166" s="54" t="n">
         <v>5</v>
@@ -52970,7 +52970,7 @@
         <v>330000</v>
       </c>
       <c r="X167" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y167" s="54" t="n">
         <v>5</v>
@@ -53279,7 +53279,7 @@
         <v>330000</v>
       </c>
       <c r="X168" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y168" s="54" t="n">
         <v>5</v>
@@ -53588,7 +53588,7 @@
         <v>330000</v>
       </c>
       <c r="X169" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y169" s="54" t="n">
         <v>5</v>
@@ -53897,7 +53897,7 @@
         <v>330000</v>
       </c>
       <c r="X170" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y170" s="54" t="n">
         <v>5</v>
@@ -54206,7 +54206,7 @@
         <v>660000</v>
       </c>
       <c r="X171" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y171" s="54" t="n">
         <v>10</v>
@@ -54515,7 +54515,7 @@
         <v>330000</v>
       </c>
       <c r="X172" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y172" s="54" t="n">
         <v>5</v>
@@ -54824,7 +54824,7 @@
         <v>330000</v>
       </c>
       <c r="X173" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y173" s="54" t="n">
         <v>5</v>
@@ -55133,7 +55133,7 @@
         <v>330000</v>
       </c>
       <c r="X174" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y174" s="54" t="n">
         <v>5</v>
@@ -55442,7 +55442,7 @@
         <v>330000</v>
       </c>
       <c r="X175" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y175" s="54" t="n">
         <v>5</v>
@@ -55751,7 +55751,7 @@
         <v>660000</v>
       </c>
       <c r="X176" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y176" s="54" t="n">
         <v>10</v>
@@ -56060,7 +56060,7 @@
         <v>330000</v>
       </c>
       <c r="X177" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y177" s="54" t="n">
         <v>5</v>
@@ -56369,7 +56369,7 @@
         <v>330000</v>
       </c>
       <c r="X178" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y178" s="54" t="n">
         <v>5</v>
@@ -56678,7 +56678,7 @@
         <v>330000</v>
       </c>
       <c r="X179" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y179" s="54" t="n">
         <v>5</v>
@@ -56987,7 +56987,7 @@
         <v>330000</v>
       </c>
       <c r="X180" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y180" s="54" t="n">
         <v>5</v>
@@ -57296,7 +57296,7 @@
         <v>330000</v>
       </c>
       <c r="X181" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y181" s="54" t="n">
         <v>5</v>
@@ -57605,7 +57605,7 @@
         <v>330000</v>
       </c>
       <c r="X182" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y182" s="54" t="n">
         <v>5</v>
@@ -57914,7 +57914,7 @@
         <v>330000</v>
       </c>
       <c r="X183" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y183" s="54" t="n">
         <v>5</v>
@@ -58223,7 +58223,7 @@
         <v>660000</v>
       </c>
       <c r="X184" s="54" t="n">
-        <v>33000</v>
+        <v>19800</v>
       </c>
       <c r="Y184" s="54" t="n">
         <v>10</v>
@@ -58532,7 +58532,7 @@
         <v>330000</v>
       </c>
       <c r="X185" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y185" s="54" t="n">
         <v>5</v>
@@ -58841,7 +58841,7 @@
         <v>330000</v>
       </c>
       <c r="X186" s="54" t="n">
-        <v>16500</v>
+        <v>9900</v>
       </c>
       <c r="Y186" s="54" t="n">
         <v>5</v>

</xml_diff>